<commit_message>
switched barrel plug for #8. touched up schematic, DRC, generated BOM, generated Gerbers
</commit_message>
<xml_diff>
--- a/manufacturing files/blockaxe1 BOM.xlsx
+++ b/manufacturing files/blockaxe1 BOM.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/skot/Work/Bitcoin/blockaxe/blockaxe1/manufacturing files/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2C75EBFA-C6F4-0646-BABB-47DACFDB4A97}" xr6:coauthVersionLast="46" xr6:coauthVersionMax="46" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6F08C3CC-8E81-C44B-8D2E-74A75BABB1DF}" xr6:coauthVersionLast="46" xr6:coauthVersionMax="46" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="240" yWindow="500" windowWidth="24240" windowHeight="25380" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="240" yWindow="500" windowWidth="30760" windowHeight="27220" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="BOM" sheetId="1" r:id="rId1"/>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="332" uniqueCount="211">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="320" uniqueCount="203">
   <si>
     <t>Qty</t>
   </si>
@@ -41,7 +41,7 @@
     <t>DNP</t>
   </si>
   <si>
-    <t>C1, C3, C4, C5, C6, C7, C8, C9, C10, C13, C14, C20, C25, C26, C47, C48</t>
+    <t>C1, C3, C4, C5, C6, C7, C10, C13, C20, C25, C26, C27, C28, C47, C48</t>
   </si>
   <si>
     <t>0.1uF</t>
@@ -65,7 +65,7 @@
     <t>CL05A475MP5NRNC</t>
   </si>
   <si>
-    <t>C11, C12, C15, C16, C17, C22, C23, C45, C46, C49, C50</t>
+    <t>C12, C15, C16, C17, C22, C23, C45, C46, C49, C50</t>
   </si>
   <si>
     <t>1uF</t>
@@ -239,12 +239,6 @@
     <t>893-1188-1-ND</t>
   </si>
   <si>
-    <t>J1, J2</t>
-  </si>
-  <si>
-    <t>TC2030-IDC</t>
-  </si>
-  <si>
     <t>J4</t>
   </si>
   <si>
@@ -260,10 +254,10 @@
     <t>J5</t>
   </si>
   <si>
-    <t>PJ-002B</t>
-  </si>
-  <si>
-    <t>CP-002B-ND</t>
+    <t>EJ503A</t>
+  </si>
+  <si>
+    <t>EJ503A-ND</t>
   </si>
   <si>
     <t>J6</t>
@@ -278,12 +272,6 @@
     <t>0470531000</t>
   </si>
   <si>
-    <t>J7</t>
-  </si>
-  <si>
-    <t>Conn_01x03</t>
-  </si>
-  <si>
     <t>L2</t>
   </si>
   <si>
@@ -374,19 +362,31 @@
     <t>RC0402FR-071ML</t>
   </si>
   <si>
-    <t>R11</t>
-  </si>
-  <si>
-    <t>78.7k 1%</t>
-  </si>
-  <si>
-    <t>311-78.7KLRCT-ND</t>
-  </si>
-  <si>
-    <t>RC0402FR-0778K7L</t>
-  </si>
-  <si>
-    <t>R16, R18</t>
+    <t>R13, R28</t>
+  </si>
+  <si>
+    <t>20k</t>
+  </si>
+  <si>
+    <t>311-20.0KLRCT-ND</t>
+  </si>
+  <si>
+    <t>RC0402FR-0720KL</t>
+  </si>
+  <si>
+    <t>R17</t>
+  </si>
+  <si>
+    <t>130k 1%</t>
+  </si>
+  <si>
+    <t>YAG2969CT-ND</t>
+  </si>
+  <si>
+    <t>RC0402FR-07130KL</t>
+  </si>
+  <si>
+    <t>R18</t>
   </si>
   <si>
     <t>182k 1%</t>
@@ -398,18 +398,6 @@
     <t>RC0402FR-07182KL</t>
   </si>
   <si>
-    <t>R17</t>
-  </si>
-  <si>
-    <t>130k 1%</t>
-  </si>
-  <si>
-    <t>YAG2969CT-ND</t>
-  </si>
-  <si>
-    <t>RC0402FR-07130KL</t>
-  </si>
-  <si>
     <t>R19</t>
   </si>
   <si>
@@ -485,18 +473,6 @@
     <t>RC0402FR-072K67L</t>
   </si>
   <si>
-    <t>R28</t>
-  </si>
-  <si>
-    <t>20k</t>
-  </si>
-  <si>
-    <t>P20.0KLCT-ND</t>
-  </si>
-  <si>
-    <t>ERJ-2RKF2002X</t>
-  </si>
-  <si>
     <t>R29</t>
   </si>
   <si>
@@ -524,18 +500,15 @@
     <t>SW1, SW2</t>
   </si>
   <si>
-    <t>EVQ-9P701P</t>
-  </si>
-  <si>
-    <t>P19095CT-ND</t>
+    <t>TL3330AF260QG</t>
+  </si>
+  <si>
+    <t>EG4389CT-ND</t>
   </si>
   <si>
     <t>U1</t>
   </si>
   <si>
-    <t>~</t>
-  </si>
-  <si>
     <t>U2</t>
   </si>
   <si>
@@ -545,16 +518,7 @@
     <t>497-16240-ND</t>
   </si>
   <si>
-    <t>U4</t>
-  </si>
-  <si>
-    <t>TXB0104RGYR</t>
-  </si>
-  <si>
-    <t>296-21930-1-ND</t>
-  </si>
-  <si>
-    <t>U5, U6</t>
+    <t>U5</t>
   </si>
   <si>
     <t>ADP171AUJ-R7</t>
@@ -620,6 +584,18 @@
     <t>EMC2101-R-ACZL-TR</t>
   </si>
   <si>
+    <t>U12</t>
+  </si>
+  <si>
+    <t>SN74AVC4T774</t>
+  </si>
+  <si>
+    <t>296-24739-1-ND</t>
+  </si>
+  <si>
+    <t>SN74AVC4T774PWR</t>
+  </si>
+  <si>
     <t>U16</t>
   </si>
   <si>
@@ -638,10 +614,7 @@
     <t>50MHz</t>
   </si>
   <si>
-    <t>XC2889CT-ND</t>
-  </si>
-  <si>
-    <t>ECS-3225MV-500-CN-TR</t>
+    <t>SX3M50.000E20F30THN</t>
   </si>
   <si>
     <t>Y2</t>
@@ -654,6 +627,9 @@
   </si>
   <si>
     <t>SC32S-7PF20PPM</t>
+  </si>
+  <si>
+    <t>BZM2</t>
   </si>
 </sst>
 </file>
@@ -703,9 +679,15 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1044,7 +1026,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:F57"/>
+  <dimension ref="A1:F54"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="5.6640625" customWidth="1"/>
@@ -1074,7 +1056,7 @@
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A2">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B2" t="s">
         <v>6</v>
@@ -1108,7 +1090,7 @@
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A4">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B4" t="s">
         <v>14</v>
@@ -1363,7 +1345,7 @@
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A19">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B19" t="s">
         <v>72</v>
@@ -1371,19 +1353,25 @@
       <c r="C19" t="s">
         <v>73</v>
       </c>
+      <c r="D19" t="s">
+        <v>74</v>
+      </c>
+      <c r="E19" t="s">
+        <v>75</v>
+      </c>
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A20">
         <v>1</v>
       </c>
       <c r="B20" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="C20" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="D20" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="E20" t="s">
         <v>77</v>
@@ -1394,16 +1382,16 @@
         <v>1</v>
       </c>
       <c r="B21" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="C21" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="D21" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="E21" t="s">
-        <v>79</v>
+        <v>82</v>
       </c>
     </row>
     <row r="22" spans="1:5" x14ac:dyDescent="0.2">
@@ -1411,16 +1399,16 @@
         <v>1</v>
       </c>
       <c r="B22" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="C22" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="D22" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="E22" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
     </row>
     <row r="23" spans="1:5" x14ac:dyDescent="0.2">
@@ -1428,10 +1416,16 @@
         <v>1</v>
       </c>
       <c r="B23" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="C23" t="s">
-        <v>86</v>
+        <v>88</v>
+      </c>
+      <c r="D23" t="s">
+        <v>89</v>
+      </c>
+      <c r="E23" t="s">
+        <v>88</v>
       </c>
     </row>
     <row r="24" spans="1:5" x14ac:dyDescent="0.2">
@@ -1439,84 +1433,84 @@
         <v>1</v>
       </c>
       <c r="B24" t="s">
-        <v>87</v>
+        <v>90</v>
       </c>
       <c r="C24" t="s">
-        <v>88</v>
+        <v>91</v>
       </c>
       <c r="D24" t="s">
-        <v>89</v>
+        <v>92</v>
       </c>
       <c r="E24" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
     </row>
     <row r="25" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A25">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="B25" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="C25" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="D25" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="E25" t="s">
-        <v>92</v>
+        <v>96</v>
       </c>
     </row>
     <row r="26" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A26">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="B26" t="s">
-        <v>94</v>
+        <v>97</v>
       </c>
       <c r="C26" t="s">
-        <v>95</v>
+        <v>98</v>
       </c>
       <c r="D26" t="s">
-        <v>96</v>
+        <v>99</v>
       </c>
       <c r="E26" t="s">
-        <v>95</v>
+        <v>100</v>
       </c>
     </row>
     <row r="27" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A27">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="B27" t="s">
-        <v>97</v>
+        <v>101</v>
       </c>
       <c r="C27" t="s">
-        <v>98</v>
+        <v>102</v>
       </c>
       <c r="D27" t="s">
-        <v>99</v>
+        <v>103</v>
       </c>
       <c r="E27" t="s">
-        <v>100</v>
+        <v>104</v>
       </c>
     </row>
     <row r="28" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A28">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B28" t="s">
-        <v>101</v>
+        <v>105</v>
       </c>
       <c r="C28" t="s">
-        <v>102</v>
+        <v>106</v>
       </c>
       <c r="D28" t="s">
-        <v>103</v>
+        <v>107</v>
       </c>
       <c r="E28" t="s">
-        <v>104</v>
+        <v>108</v>
       </c>
     </row>
     <row r="29" spans="1:5" x14ac:dyDescent="0.2">
@@ -1524,33 +1518,33 @@
         <v>1</v>
       </c>
       <c r="B29" t="s">
-        <v>105</v>
+        <v>109</v>
       </c>
       <c r="C29" t="s">
-        <v>106</v>
+        <v>110</v>
       </c>
       <c r="D29" t="s">
-        <v>107</v>
+        <v>111</v>
       </c>
       <c r="E29" t="s">
-        <v>108</v>
+        <v>112</v>
       </c>
     </row>
     <row r="30" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A30">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="B30" t="s">
-        <v>109</v>
+        <v>113</v>
       </c>
       <c r="C30" t="s">
-        <v>110</v>
+        <v>114</v>
       </c>
       <c r="D30" t="s">
-        <v>111</v>
+        <v>115</v>
       </c>
       <c r="E30" t="s">
-        <v>112</v>
+        <v>116</v>
       </c>
     </row>
     <row r="31" spans="1:5" x14ac:dyDescent="0.2">
@@ -1558,16 +1552,16 @@
         <v>1</v>
       </c>
       <c r="B31" t="s">
-        <v>113</v>
+        <v>117</v>
       </c>
       <c r="C31" t="s">
-        <v>114</v>
+        <v>118</v>
       </c>
       <c r="D31" t="s">
-        <v>115</v>
+        <v>119</v>
       </c>
       <c r="E31" t="s">
-        <v>116</v>
+        <v>120</v>
       </c>
     </row>
     <row r="32" spans="1:5" x14ac:dyDescent="0.2">
@@ -1575,33 +1569,33 @@
         <v>1</v>
       </c>
       <c r="B32" t="s">
-        <v>117</v>
+        <v>121</v>
       </c>
       <c r="C32" t="s">
-        <v>118</v>
+        <v>122</v>
       </c>
       <c r="D32" t="s">
-        <v>119</v>
+        <v>123</v>
       </c>
       <c r="E32" t="s">
-        <v>120</v>
+        <v>124</v>
       </c>
     </row>
     <row r="33" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A33">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B33" t="s">
-        <v>121</v>
+        <v>125</v>
       </c>
       <c r="C33" t="s">
-        <v>122</v>
+        <v>126</v>
       </c>
       <c r="D33" t="s">
-        <v>123</v>
+        <v>127</v>
       </c>
       <c r="E33" t="s">
-        <v>124</v>
+        <v>128</v>
       </c>
     </row>
     <row r="34" spans="1:6" x14ac:dyDescent="0.2">
@@ -1609,7 +1603,7 @@
         <v>1</v>
       </c>
       <c r="B34" t="s">
-        <v>125</v>
+        <v>129</v>
       </c>
       <c r="C34" t="s">
         <v>126</v>
@@ -1620,22 +1614,25 @@
       <c r="E34" t="s">
         <v>128</v>
       </c>
+      <c r="F34" t="s">
+        <v>5</v>
+      </c>
     </row>
     <row r="35" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A35">
         <v>1</v>
       </c>
       <c r="B35" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="C35" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="D35" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="E35" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
     </row>
     <row r="36" spans="1:6" x14ac:dyDescent="0.2">
@@ -1643,19 +1640,16 @@
         <v>1</v>
       </c>
       <c r="B36" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="C36" t="s">
-        <v>130</v>
+        <v>135</v>
       </c>
       <c r="D36" t="s">
-        <v>131</v>
+        <v>136</v>
       </c>
       <c r="E36" t="s">
-        <v>132</v>
-      </c>
-      <c r="F36" t="s">
-        <v>5</v>
+        <v>137</v>
       </c>
     </row>
     <row r="37" spans="1:6" x14ac:dyDescent="0.2">
@@ -1663,33 +1657,33 @@
         <v>1</v>
       </c>
       <c r="B37" t="s">
-        <v>134</v>
+        <v>138</v>
       </c>
       <c r="C37" t="s">
-        <v>135</v>
+        <v>139</v>
       </c>
       <c r="D37" t="s">
-        <v>136</v>
+        <v>140</v>
       </c>
       <c r="E37" t="s">
-        <v>137</v>
+        <v>141</v>
       </c>
     </row>
     <row r="38" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A38">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="B38" t="s">
-        <v>138</v>
+        <v>142</v>
       </c>
       <c r="C38" t="s">
-        <v>139</v>
+        <v>143</v>
       </c>
       <c r="D38" t="s">
-        <v>140</v>
+        <v>144</v>
       </c>
       <c r="E38" t="s">
-        <v>141</v>
+        <v>145</v>
       </c>
     </row>
     <row r="39" spans="1:6" x14ac:dyDescent="0.2">
@@ -1697,33 +1691,33 @@
         <v>1</v>
       </c>
       <c r="B39" t="s">
-        <v>142</v>
+        <v>146</v>
       </c>
       <c r="C39" t="s">
-        <v>143</v>
+        <v>147</v>
       </c>
       <c r="D39" t="s">
-        <v>144</v>
+        <v>148</v>
       </c>
       <c r="E39" t="s">
-        <v>145</v>
+        <v>149</v>
       </c>
     </row>
     <row r="40" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A40">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B40" t="s">
-        <v>146</v>
+        <v>150</v>
       </c>
       <c r="C40" t="s">
-        <v>147</v>
+        <v>151</v>
       </c>
       <c r="D40" t="s">
-        <v>148</v>
+        <v>152</v>
       </c>
       <c r="E40" t="s">
-        <v>149</v>
+        <v>153</v>
       </c>
     </row>
     <row r="41" spans="1:6" x14ac:dyDescent="0.2">
@@ -1731,33 +1725,33 @@
         <v>1</v>
       </c>
       <c r="B41" t="s">
-        <v>150</v>
+        <v>154</v>
       </c>
       <c r="C41" t="s">
-        <v>151</v>
+        <v>155</v>
       </c>
       <c r="D41" t="s">
-        <v>152</v>
+        <v>156</v>
       </c>
       <c r="E41" t="s">
-        <v>153</v>
+        <v>157</v>
       </c>
     </row>
     <row r="42" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A42">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="B42" t="s">
-        <v>154</v>
+        <v>158</v>
       </c>
       <c r="C42" t="s">
-        <v>155</v>
+        <v>159</v>
       </c>
       <c r="D42" t="s">
-        <v>156</v>
+        <v>160</v>
       </c>
       <c r="E42" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
     </row>
     <row r="43" spans="1:6" x14ac:dyDescent="0.2">
@@ -1765,16 +1759,10 @@
         <v>1</v>
       </c>
       <c r="B43" t="s">
-        <v>158</v>
-      </c>
-      <c r="C43" t="s">
-        <v>159</v>
-      </c>
-      <c r="D43" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="E43" t="s">
-        <v>161</v>
+        <v>202</v>
       </c>
     </row>
     <row r="44" spans="1:6" x14ac:dyDescent="0.2">
@@ -1791,24 +1779,24 @@
         <v>164</v>
       </c>
       <c r="E44" t="s">
-        <v>165</v>
+        <v>163</v>
       </c>
     </row>
     <row r="45" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A45">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B45" t="s">
+        <v>165</v>
+      </c>
+      <c r="C45" t="s">
         <v>166</v>
       </c>
-      <c r="C45" t="s">
+      <c r="D45" t="s">
         <v>167</v>
       </c>
-      <c r="D45" t="s">
+      <c r="E45" t="s">
         <v>168</v>
-      </c>
-      <c r="E45" t="s">
-        <v>167</v>
       </c>
     </row>
     <row r="46" spans="1:6" x14ac:dyDescent="0.2">
@@ -1821,22 +1809,28 @@
       <c r="C46" t="s">
         <v>170</v>
       </c>
+      <c r="D46" t="s">
+        <v>171</v>
+      </c>
+      <c r="E46" t="s">
+        <v>170</v>
+      </c>
     </row>
     <row r="47" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A47">
         <v>1</v>
       </c>
       <c r="B47" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="C47" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="D47" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="E47" t="s">
-        <v>172</v>
+        <v>175</v>
       </c>
     </row>
     <row r="48" spans="1:6" x14ac:dyDescent="0.2">
@@ -1844,33 +1838,33 @@
         <v>1</v>
       </c>
       <c r="B48" t="s">
-        <v>174</v>
+        <v>176</v>
       </c>
       <c r="C48" t="s">
-        <v>175</v>
+        <v>177</v>
       </c>
       <c r="D48" t="s">
-        <v>176</v>
+        <v>178</v>
       </c>
       <c r="E48" t="s">
-        <v>175</v>
+        <v>179</v>
       </c>
     </row>
     <row r="49" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A49">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B49" t="s">
-        <v>177</v>
+        <v>180</v>
       </c>
       <c r="C49" t="s">
-        <v>178</v>
+        <v>181</v>
       </c>
       <c r="D49" t="s">
-        <v>179</v>
+        <v>182</v>
       </c>
       <c r="E49" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
     </row>
     <row r="50" spans="1:5" x14ac:dyDescent="0.2">
@@ -1878,16 +1872,16 @@
         <v>1</v>
       </c>
       <c r="B50" t="s">
-        <v>181</v>
+        <v>183</v>
       </c>
       <c r="C50" t="s">
-        <v>182</v>
+        <v>184</v>
       </c>
       <c r="D50" t="s">
-        <v>183</v>
+        <v>185</v>
       </c>
       <c r="E50" t="s">
-        <v>182</v>
+        <v>186</v>
       </c>
     </row>
     <row r="51" spans="1:5" x14ac:dyDescent="0.2">
@@ -1895,16 +1889,16 @@
         <v>1</v>
       </c>
       <c r="B51" t="s">
-        <v>184</v>
+        <v>187</v>
       </c>
       <c r="C51" t="s">
-        <v>185</v>
+        <v>188</v>
       </c>
       <c r="D51" t="s">
-        <v>186</v>
+        <v>189</v>
       </c>
       <c r="E51" t="s">
-        <v>187</v>
+        <v>190</v>
       </c>
     </row>
     <row r="52" spans="1:5" x14ac:dyDescent="0.2">
@@ -1912,16 +1906,16 @@
         <v>1</v>
       </c>
       <c r="B52" t="s">
-        <v>188</v>
+        <v>191</v>
       </c>
       <c r="C52" t="s">
-        <v>189</v>
+        <v>192</v>
       </c>
       <c r="D52" t="s">
-        <v>190</v>
+        <v>193</v>
       </c>
       <c r="E52" t="s">
-        <v>191</v>
+        <v>194</v>
       </c>
     </row>
     <row r="53" spans="1:5" x14ac:dyDescent="0.2">
@@ -1929,16 +1923,13 @@
         <v>1</v>
       </c>
       <c r="B53" t="s">
-        <v>192</v>
+        <v>195</v>
       </c>
       <c r="C53" t="s">
-        <v>193</v>
-      </c>
-      <c r="D53" t="s">
-        <v>194</v>
+        <v>196</v>
       </c>
       <c r="E53" t="s">
-        <v>193</v>
+        <v>197</v>
       </c>
     </row>
     <row r="54" spans="1:5" x14ac:dyDescent="0.2">
@@ -1946,67 +1937,16 @@
         <v>1</v>
       </c>
       <c r="B54" t="s">
-        <v>195</v>
+        <v>198</v>
       </c>
       <c r="C54" t="s">
-        <v>196</v>
+        <v>199</v>
       </c>
       <c r="D54" t="s">
-        <v>197</v>
+        <v>200</v>
       </c>
       <c r="E54" t="s">
-        <v>198</v>
-      </c>
-    </row>
-    <row r="55" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A55">
-        <v>1</v>
-      </c>
-      <c r="B55" t="s">
-        <v>199</v>
-      </c>
-      <c r="C55" t="s">
-        <v>200</v>
-      </c>
-      <c r="D55" t="s">
         <v>201</v>
-      </c>
-      <c r="E55" t="s">
-        <v>202</v>
-      </c>
-    </row>
-    <row r="56" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A56">
-        <v>1</v>
-      </c>
-      <c r="B56" t="s">
-        <v>203</v>
-      </c>
-      <c r="C56" t="s">
-        <v>204</v>
-      </c>
-      <c r="D56" t="s">
-        <v>205</v>
-      </c>
-      <c r="E56" t="s">
-        <v>206</v>
-      </c>
-    </row>
-    <row r="57" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A57">
-        <v>1</v>
-      </c>
-      <c r="B57" t="s">
-        <v>207</v>
-      </c>
-      <c r="C57" t="s">
-        <v>208</v>
-      </c>
-      <c r="D57" t="s">
-        <v>209</v>
-      </c>
-      <c r="E57" t="s">
-        <v>210</v>
       </c>
     </row>
   </sheetData>
@@ -2016,594 +1956,581 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:C53"/>
+  <dimension ref="A1:C52"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="5.6640625" customWidth="1"/>
-    <col min="2" max="4" width="30.6640625" customWidth="1"/>
+    <col min="2" max="2" width="30.6640625" style="3" customWidth="1"/>
+    <col min="3" max="4" width="30.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:3" ht="16" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" s="2" t="s">
         <v>1</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:3" ht="32" x14ac:dyDescent="0.2">
       <c r="A2">
-        <v>16</v>
-      </c>
-      <c r="B2" t="s">
+        <v>15</v>
+      </c>
+      <c r="B2" s="3" t="s">
         <v>6</v>
       </c>
       <c r="C2" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:3" ht="16" x14ac:dyDescent="0.2">
       <c r="A3">
         <v>1</v>
       </c>
-      <c r="B3" t="s">
+      <c r="B3" s="3" t="s">
         <v>10</v>
       </c>
       <c r="C3" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:3" ht="32" x14ac:dyDescent="0.2">
       <c r="A4">
-        <v>11</v>
-      </c>
-      <c r="B4" t="s">
+        <v>10</v>
+      </c>
+      <c r="B4" s="3" t="s">
         <v>14</v>
       </c>
       <c r="C4" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:3" ht="16" x14ac:dyDescent="0.2">
       <c r="A5">
         <v>1</v>
       </c>
-      <c r="B5" t="s">
+      <c r="B5" s="3" t="s">
         <v>18</v>
       </c>
       <c r="C5" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:3" ht="16" x14ac:dyDescent="0.2">
       <c r="A6">
         <v>2</v>
       </c>
-      <c r="B6" t="s">
+      <c r="B6" s="3" t="s">
         <v>22</v>
       </c>
       <c r="C6" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:3" ht="16" x14ac:dyDescent="0.2">
       <c r="A7">
         <v>1</v>
       </c>
-      <c r="B7" t="s">
+      <c r="B7" s="3" t="s">
         <v>26</v>
       </c>
       <c r="C7" t="s">
         <v>28</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:3" ht="16" x14ac:dyDescent="0.2">
       <c r="A8">
         <v>3</v>
       </c>
-      <c r="B8" t="s">
+      <c r="B8" s="3" t="s">
         <v>30</v>
       </c>
       <c r="C8" t="s">
         <v>32</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:3" ht="16" x14ac:dyDescent="0.2">
       <c r="A9">
         <v>1</v>
       </c>
-      <c r="B9" t="s">
+      <c r="B9" s="3" t="s">
         <v>34</v>
       </c>
       <c r="C9" t="s">
         <v>36</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:3" ht="16" x14ac:dyDescent="0.2">
       <c r="A10">
         <v>2</v>
       </c>
-      <c r="B10" t="s">
+      <c r="B10" s="3" t="s">
         <v>38</v>
       </c>
       <c r="C10" t="s">
         <v>39</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:3" ht="16" x14ac:dyDescent="0.2">
       <c r="A11">
         <v>2</v>
       </c>
-      <c r="B11" t="s">
+      <c r="B11" s="3" t="s">
         <v>41</v>
       </c>
       <c r="C11" t="s">
         <v>43</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:3" ht="16" x14ac:dyDescent="0.2">
       <c r="A12">
         <v>1</v>
       </c>
-      <c r="B12" t="s">
+      <c r="B12" s="3" t="s">
         <v>45</v>
       </c>
       <c r="C12" t="s">
         <v>47</v>
       </c>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:3" ht="16" x14ac:dyDescent="0.2">
       <c r="A13">
         <v>1</v>
       </c>
-      <c r="B13" t="s">
+      <c r="B13" s="3" t="s">
         <v>49</v>
       </c>
       <c r="C13" t="s">
         <v>51</v>
       </c>
     </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:3" ht="16" x14ac:dyDescent="0.2">
       <c r="A14">
         <v>1</v>
       </c>
-      <c r="B14" t="s">
+      <c r="B14" s="3" t="s">
         <v>53</v>
       </c>
       <c r="C14" t="s">
         <v>55</v>
       </c>
     </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:3" ht="16" x14ac:dyDescent="0.2">
       <c r="A15">
         <v>1</v>
       </c>
-      <c r="B15" t="s">
+      <c r="B15" s="3" t="s">
         <v>57</v>
       </c>
       <c r="C15" t="s">
         <v>59</v>
       </c>
     </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:3" ht="16" x14ac:dyDescent="0.2">
       <c r="A16">
         <v>1</v>
       </c>
-      <c r="B16" t="s">
+      <c r="B16" s="3" t="s">
         <v>61</v>
       </c>
       <c r="C16" t="s">
         <v>63</v>
       </c>
     </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:3" ht="16" x14ac:dyDescent="0.2">
       <c r="A17">
         <v>1</v>
       </c>
-      <c r="B17" t="s">
+      <c r="B17" s="3" t="s">
         <v>65</v>
       </c>
       <c r="C17" t="s">
         <v>67</v>
       </c>
     </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:3" ht="16" x14ac:dyDescent="0.2">
       <c r="A18">
         <v>1</v>
       </c>
-      <c r="B18" t="s">
+      <c r="B18" s="3" t="s">
         <v>69</v>
       </c>
       <c r="C18" t="s">
         <v>71</v>
       </c>
     </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:3" ht="16" x14ac:dyDescent="0.2">
       <c r="A19">
         <v>1</v>
       </c>
-      <c r="B19" t="s">
+      <c r="B19" s="3" t="s">
+        <v>72</v>
+      </c>
+      <c r="C19" t="s">
         <v>74</v>
       </c>
-      <c r="C19" t="s">
+    </row>
+    <row r="20" spans="1:3" ht="16" x14ac:dyDescent="0.2">
+      <c r="A20">
+        <v>1</v>
+      </c>
+      <c r="B20" s="3" t="s">
         <v>76</v>
       </c>
-    </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A20">
-        <v>1</v>
-      </c>
-      <c r="B20" t="s">
+      <c r="C20" t="s">
         <v>78</v>
       </c>
-      <c r="C20" t="s">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.2">
+    </row>
+    <row r="21" spans="1:3" ht="16" x14ac:dyDescent="0.2">
       <c r="A21">
         <v>1</v>
       </c>
-      <c r="B21" t="s">
+      <c r="B21" s="3" t="s">
+        <v>79</v>
+      </c>
+      <c r="C21" t="s">
         <v>81</v>
       </c>
-      <c r="C21" t="s">
+    </row>
+    <row r="22" spans="1:3" ht="16" x14ac:dyDescent="0.2">
+      <c r="A22">
+        <v>1</v>
+      </c>
+      <c r="B22" s="3" t="s">
         <v>83</v>
       </c>
-    </row>
-    <row r="22" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A22">
-        <v>1</v>
-      </c>
-      <c r="B22" t="s">
+      <c r="C22" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="23" spans="1:3" ht="16" x14ac:dyDescent="0.2">
+      <c r="A23">
+        <v>1</v>
+      </c>
+      <c r="B23" s="3" t="s">
         <v>87</v>
       </c>
-      <c r="C22" t="s">
+      <c r="C23" t="s">
         <v>89</v>
       </c>
     </row>
-    <row r="23" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A23">
-        <v>1</v>
-      </c>
-      <c r="B23" t="s">
-        <v>91</v>
-      </c>
-      <c r="C23" t="s">
-        <v>93</v>
-      </c>
-    </row>
-    <row r="24" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:3" ht="16" x14ac:dyDescent="0.2">
       <c r="A24">
         <v>1</v>
       </c>
-      <c r="B24" t="s">
-        <v>94</v>
+      <c r="B24" s="3" t="s">
+        <v>90</v>
       </c>
       <c r="C24" t="s">
-        <v>96</v>
-      </c>
-    </row>
-    <row r="25" spans="1:3" x14ac:dyDescent="0.2">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="25" spans="1:3" ht="16" x14ac:dyDescent="0.2">
       <c r="A25">
         <v>6</v>
       </c>
-      <c r="B25" t="s">
-        <v>97</v>
+      <c r="B25" s="3" t="s">
+        <v>93</v>
       </c>
       <c r="C25" t="s">
-        <v>99</v>
-      </c>
-    </row>
-    <row r="26" spans="1:3" x14ac:dyDescent="0.2">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="26" spans="1:3" ht="16" x14ac:dyDescent="0.2">
       <c r="A26">
         <v>2</v>
       </c>
-      <c r="B26" t="s">
+      <c r="B26" s="3" t="s">
+        <v>97</v>
+      </c>
+      <c r="C26" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="27" spans="1:3" ht="16" x14ac:dyDescent="0.2">
+      <c r="A27">
+        <v>1</v>
+      </c>
+      <c r="B27" s="3" t="s">
         <v>101</v>
       </c>
-      <c r="C26" t="s">
+      <c r="C27" t="s">
         <v>103</v>
       </c>
     </row>
-    <row r="27" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A27">
-        <v>1</v>
-      </c>
-      <c r="B27" t="s">
+    <row r="28" spans="1:3" ht="16" x14ac:dyDescent="0.2">
+      <c r="A28">
+        <v>1</v>
+      </c>
+      <c r="B28" s="3" t="s">
         <v>105</v>
       </c>
-      <c r="C27" t="s">
+      <c r="C28" t="s">
         <v>107</v>
       </c>
     </row>
-    <row r="28" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A28">
-        <v>1</v>
-      </c>
-      <c r="B28" t="s">
+    <row r="29" spans="1:3" ht="16" x14ac:dyDescent="0.2">
+      <c r="A29">
+        <v>1</v>
+      </c>
+      <c r="B29" s="3" t="s">
         <v>109</v>
       </c>
-      <c r="C28" t="s">
+      <c r="C29" t="s">
         <v>111</v>
       </c>
     </row>
-    <row r="29" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A29">
-        <v>1</v>
-      </c>
-      <c r="B29" t="s">
+    <row r="30" spans="1:3" ht="16" x14ac:dyDescent="0.2">
+      <c r="A30">
+        <v>2</v>
+      </c>
+      <c r="B30" s="3" t="s">
         <v>113</v>
       </c>
-      <c r="C29" t="s">
+      <c r="C30" t="s">
         <v>115</v>
       </c>
     </row>
-    <row r="30" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A30">
-        <v>1</v>
-      </c>
-      <c r="B30" t="s">
+    <row r="31" spans="1:3" ht="16" x14ac:dyDescent="0.2">
+      <c r="A31">
+        <v>1</v>
+      </c>
+      <c r="B31" s="3" t="s">
         <v>117</v>
       </c>
-      <c r="C30" t="s">
+      <c r="C31" t="s">
         <v>119</v>
       </c>
     </row>
-    <row r="31" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A31">
-        <v>2</v>
-      </c>
-      <c r="B31" t="s">
+    <row r="32" spans="1:3" ht="16" x14ac:dyDescent="0.2">
+      <c r="A32">
+        <v>1</v>
+      </c>
+      <c r="B32" s="3" t="s">
         <v>121</v>
       </c>
-      <c r="C31" t="s">
+      <c r="C32" t="s">
         <v>123</v>
       </c>
     </row>
-    <row r="32" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A32">
-        <v>1</v>
-      </c>
-      <c r="B32" t="s">
+    <row r="33" spans="1:3" ht="16" x14ac:dyDescent="0.2">
+      <c r="A33">
+        <v>1</v>
+      </c>
+      <c r="B33" s="3" t="s">
         <v>125</v>
       </c>
-      <c r="C32" t="s">
+      <c r="C33" t="s">
         <v>127</v>
       </c>
     </row>
-    <row r="33" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A33">
-        <v>1</v>
-      </c>
-      <c r="B33" t="s">
-        <v>129</v>
-      </c>
-      <c r="C33" t="s">
-        <v>131</v>
-      </c>
-    </row>
-    <row r="34" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="34" spans="1:3" ht="16" x14ac:dyDescent="0.2">
       <c r="A34">
         <v>1</v>
       </c>
-      <c r="B34" t="s">
+      <c r="B34" s="3" t="s">
+        <v>130</v>
+      </c>
+      <c r="C34" t="s">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="35" spans="1:3" ht="16" x14ac:dyDescent="0.2">
+      <c r="A35">
+        <v>1</v>
+      </c>
+      <c r="B35" s="3" t="s">
         <v>134</v>
       </c>
-      <c r="C34" t="s">
+      <c r="C35" t="s">
         <v>136</v>
       </c>
     </row>
-    <row r="35" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A35">
-        <v>1</v>
-      </c>
-      <c r="B35" t="s">
+    <row r="36" spans="1:3" ht="16" x14ac:dyDescent="0.2">
+      <c r="A36">
+        <v>1</v>
+      </c>
+      <c r="B36" s="3" t="s">
         <v>138</v>
       </c>
-      <c r="C35" t="s">
+      <c r="C36" t="s">
         <v>140</v>
       </c>
     </row>
-    <row r="36" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A36">
-        <v>1</v>
-      </c>
-      <c r="B36" t="s">
-        <v>142</v>
-      </c>
-      <c r="C36" t="s">
-        <v>144</v>
-      </c>
-    </row>
-    <row r="37" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="37" spans="1:3" ht="16" x14ac:dyDescent="0.2">
       <c r="A37">
         <v>2</v>
       </c>
-      <c r="B37" t="s">
+      <c r="B37" s="3" t="s">
+        <v>142</v>
+      </c>
+      <c r="C37" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="38" spans="1:3" ht="16" x14ac:dyDescent="0.2">
+      <c r="A38">
+        <v>1</v>
+      </c>
+      <c r="B38" s="3" t="s">
         <v>146</v>
       </c>
-      <c r="C37" t="s">
+      <c r="C38" t="s">
         <v>148</v>
       </c>
     </row>
-    <row r="38" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A38">
-        <v>1</v>
-      </c>
-      <c r="B38" t="s">
+    <row r="39" spans="1:3" ht="16" x14ac:dyDescent="0.2">
+      <c r="A39">
+        <v>1</v>
+      </c>
+      <c r="B39" s="3" t="s">
         <v>150</v>
       </c>
-      <c r="C38" t="s">
+      <c r="C39" t="s">
         <v>152</v>
       </c>
     </row>
-    <row r="39" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A39">
-        <v>1</v>
-      </c>
-      <c r="B39" t="s">
+    <row r="40" spans="1:3" ht="16" x14ac:dyDescent="0.2">
+      <c r="A40">
+        <v>1</v>
+      </c>
+      <c r="B40" s="3" t="s">
         <v>154</v>
       </c>
-      <c r="C39" t="s">
+      <c r="C40" t="s">
         <v>156</v>
       </c>
     </row>
-    <row r="40" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A40">
-        <v>1</v>
-      </c>
-      <c r="B40" t="s">
+    <row r="41" spans="1:3" ht="16" x14ac:dyDescent="0.2">
+      <c r="A41">
+        <v>2</v>
+      </c>
+      <c r="B41" s="3" t="s">
         <v>158</v>
       </c>
-      <c r="C40" t="s">
+      <c r="C41" t="s">
         <v>160</v>
       </c>
     </row>
-    <row r="41" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A41">
-        <v>1</v>
-      </c>
-      <c r="B41" t="s">
+    <row r="42" spans="1:3" ht="16" x14ac:dyDescent="0.2">
+      <c r="A42">
+        <v>1</v>
+      </c>
+      <c r="B42" s="3" t="s">
         <v>162</v>
       </c>
-      <c r="C41" t="s">
+      <c r="C42" t="s">
         <v>164</v>
       </c>
     </row>
-    <row r="42" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A42">
-        <v>2</v>
-      </c>
-      <c r="B42" t="s">
-        <v>166</v>
-      </c>
-      <c r="C42" t="s">
-        <v>168</v>
-      </c>
-    </row>
-    <row r="43" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="43" spans="1:3" ht="16" x14ac:dyDescent="0.2">
       <c r="A43">
         <v>1</v>
       </c>
-      <c r="B43" t="s">
+      <c r="B43" s="3" t="s">
+        <v>165</v>
+      </c>
+      <c r="C43" t="s">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="44" spans="1:3" ht="16" x14ac:dyDescent="0.2">
+      <c r="A44">
+        <v>1</v>
+      </c>
+      <c r="B44" s="3" t="s">
+        <v>169</v>
+      </c>
+      <c r="C44" t="s">
         <v>171</v>
       </c>
-      <c r="C43" t="s">
-        <v>173</v>
-      </c>
-    </row>
-    <row r="44" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A44">
-        <v>1</v>
-      </c>
-      <c r="B44" t="s">
+    </row>
+    <row r="45" spans="1:3" ht="16" x14ac:dyDescent="0.2">
+      <c r="A45">
+        <v>1</v>
+      </c>
+      <c r="B45" s="3" t="s">
+        <v>172</v>
+      </c>
+      <c r="C45" t="s">
         <v>174</v>
       </c>
-      <c r="C44" t="s">
+    </row>
+    <row r="46" spans="1:3" ht="16" x14ac:dyDescent="0.2">
+      <c r="A46">
+        <v>1</v>
+      </c>
+      <c r="B46" s="3" t="s">
         <v>176</v>
       </c>
-    </row>
-    <row r="45" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A45">
-        <v>2</v>
-      </c>
-      <c r="B45" t="s">
-        <v>177</v>
-      </c>
-      <c r="C45" t="s">
-        <v>179</v>
-      </c>
-    </row>
-    <row r="46" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A46">
-        <v>1</v>
-      </c>
-      <c r="B46" t="s">
-        <v>181</v>
-      </c>
       <c r="C46" t="s">
+        <v>178</v>
+      </c>
+    </row>
+    <row r="47" spans="1:3" ht="16" x14ac:dyDescent="0.2">
+      <c r="A47">
+        <v>1</v>
+      </c>
+      <c r="B47" s="3" t="s">
+        <v>180</v>
+      </c>
+      <c r="C47" t="s">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="48" spans="1:3" ht="16" x14ac:dyDescent="0.2">
+      <c r="A48">
+        <v>1</v>
+      </c>
+      <c r="B48" s="3" t="s">
         <v>183</v>
       </c>
-    </row>
-    <row r="47" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A47">
-        <v>1</v>
-      </c>
-      <c r="B47" t="s">
-        <v>184</v>
-      </c>
-      <c r="C47" t="s">
-        <v>186</v>
-      </c>
-    </row>
-    <row r="48" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A48">
-        <v>1</v>
-      </c>
-      <c r="B48" t="s">
-        <v>188</v>
-      </c>
       <c r="C48" t="s">
-        <v>190</v>
-      </c>
-    </row>
-    <row r="49" spans="1:3" x14ac:dyDescent="0.2">
+        <v>185</v>
+      </c>
+    </row>
+    <row r="49" spans="1:3" ht="16" x14ac:dyDescent="0.2">
       <c r="A49">
         <v>1</v>
       </c>
-      <c r="B49" t="s">
-        <v>192</v>
+      <c r="B49" s="3" t="s">
+        <v>187</v>
       </c>
       <c r="C49" t="s">
-        <v>194</v>
-      </c>
-    </row>
-    <row r="50" spans="1:3" x14ac:dyDescent="0.2">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="50" spans="1:3" ht="16" x14ac:dyDescent="0.2">
       <c r="A50">
         <v>1</v>
       </c>
-      <c r="B50" t="s">
+      <c r="B50" s="3" t="s">
+        <v>191</v>
+      </c>
+      <c r="C50" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="51" spans="1:3" ht="16" x14ac:dyDescent="0.2">
+      <c r="A51">
+        <v>1</v>
+      </c>
+      <c r="B51" s="3" t="s">
         <v>195</v>
       </c>
-      <c r="C50" t="s">
-        <v>197</v>
-      </c>
-    </row>
-    <row r="51" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A51">
-        <v>1</v>
-      </c>
-      <c r="B51" t="s">
-        <v>199</v>
-      </c>
-      <c r="C51" t="s">
-        <v>201</v>
-      </c>
-    </row>
-    <row r="52" spans="1:3" x14ac:dyDescent="0.2">
+    </row>
+    <row r="52" spans="1:3" ht="16" x14ac:dyDescent="0.2">
       <c r="A52">
         <v>1</v>
       </c>
-      <c r="B52" t="s">
-        <v>203</v>
+      <c r="B52" s="3" t="s">
+        <v>198</v>
       </c>
       <c r="C52" t="s">
-        <v>205</v>
-      </c>
-    </row>
-    <row r="53" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A53">
-        <v>1</v>
-      </c>
-      <c r="B53" t="s">
-        <v>207</v>
-      </c>
-      <c r="C53" t="s">
-        <v>209</v>
+        <v>200</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
added stm32 crystal for #9
</commit_message>
<xml_diff>
--- a/manufacturing files/blockaxe1 BOM.xlsx
+++ b/manufacturing files/blockaxe1 BOM.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/skot/Work/Bitcoin/blockaxe/blockaxe1/manufacturing files/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6F08C3CC-8E81-C44B-8D2E-74A75BABB1DF}" xr6:coauthVersionLast="46" xr6:coauthVersionMax="46" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{29FC904F-6887-2E44-8DD1-926F5CC7C9A9}" xr6:coauthVersionLast="46" xr6:coauthVersionMax="46" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="240" yWindow="500" windowWidth="30760" windowHeight="27220" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="240" yWindow="500" windowWidth="28500" windowHeight="25000" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="BOM" sheetId="1" r:id="rId1"/>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="320" uniqueCount="203">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="320" uniqueCount="204">
   <si>
     <t>Qty</t>
   </si>
@@ -65,6 +65,18 @@
     <t>CL05A475MP5NRNC</t>
   </si>
   <si>
+    <t>C8, C9</t>
+  </si>
+  <si>
+    <t>20pF</t>
+  </si>
+  <si>
+    <t>490-GCM1555C1H200JA16DCT-ND</t>
+  </si>
+  <si>
+    <t>GCM1555C1H200JA16D</t>
+  </si>
+  <si>
     <t>C12, C15, C16, C17, C22, C23, C45, C46, C49, C50</t>
   </si>
   <si>
@@ -218,18 +230,6 @@
     <t>CL21C221JBANNNC</t>
   </si>
   <si>
-    <t>D1</t>
-  </si>
-  <si>
-    <t>SS310</t>
-  </si>
-  <si>
-    <t>SK310A-LTPMSCT-ND</t>
-  </si>
-  <si>
-    <t>SK310A-LTP</t>
-  </si>
-  <si>
     <t>D2</t>
   </si>
   <si>
@@ -284,16 +284,7 @@
     <t>FP0805R1-R10-R</t>
   </si>
   <si>
-    <t>Q4</t>
-  </si>
-  <si>
-    <t>CSD17575Q3</t>
-  </si>
-  <si>
-    <t>296-39994-1-ND</t>
-  </si>
-  <si>
-    <t>Q5</t>
+    <t>Q1, Q5</t>
   </si>
   <si>
     <t>CSD17312Q5</t>
@@ -509,6 +500,9 @@
     <t>U1</t>
   </si>
   <si>
+    <t>~</t>
+  </si>
+  <si>
     <t>U2</t>
   </si>
   <si>
@@ -629,7 +623,16 @@
     <t>SC32S-7PF20PPM</t>
   </si>
   <si>
-    <t>BZM2</t>
+    <t>Y3</t>
+  </si>
+  <si>
+    <t>8MHz</t>
+  </si>
+  <si>
+    <t>50-ECS-80-12-33-JGN-CT-ND</t>
+  </si>
+  <si>
+    <t>ECS-80-12-33-JGN-TR</t>
   </si>
 </sst>
 </file>
@@ -679,15 +682,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1090,7 +1087,7 @@
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A4">
-        <v>10</v>
+        <v>2</v>
       </c>
       <c r="B4" t="s">
         <v>14</v>
@@ -1107,7 +1104,7 @@
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A5">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="B5" t="s">
         <v>18</v>
@@ -1124,7 +1121,7 @@
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A6">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B6" t="s">
         <v>22</v>
@@ -1141,7 +1138,7 @@
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A7">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="B7" t="s">
         <v>26</v>
@@ -1158,7 +1155,7 @@
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A8">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="B8" t="s">
         <v>30</v>
@@ -1175,7 +1172,7 @@
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A9">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="B9" t="s">
         <v>34</v>
@@ -1192,19 +1189,19 @@
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A10">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B10" t="s">
         <v>38</v>
       </c>
       <c r="C10" t="s">
-        <v>15</v>
+        <v>39</v>
       </c>
       <c r="D10" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="E10" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.2">
@@ -1212,10 +1209,10 @@
         <v>2</v>
       </c>
       <c r="B11" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="C11" t="s">
-        <v>42</v>
+        <v>19</v>
       </c>
       <c r="D11" t="s">
         <v>43</v>
@@ -1226,7 +1223,7 @@
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A12">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="B12" t="s">
         <v>45</v>
@@ -1413,7 +1410,7 @@
     </row>
     <row r="23" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A23">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="B23" t="s">
         <v>87</v>
@@ -1430,7 +1427,7 @@
     </row>
     <row r="24" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A24">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="B24" t="s">
         <v>90</v>
@@ -1442,41 +1439,41 @@
         <v>92</v>
       </c>
       <c r="E24" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
     </row>
     <row r="25" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A25">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="B25" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="C25" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="D25" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="E25" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
     </row>
     <row r="26" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A26">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B26" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="C26" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="D26" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="E26" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
     </row>
     <row r="27" spans="1:5" x14ac:dyDescent="0.2">
@@ -1484,16 +1481,16 @@
         <v>1</v>
       </c>
       <c r="B27" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="C27" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="D27" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="E27" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
     </row>
     <row r="28" spans="1:5" x14ac:dyDescent="0.2">
@@ -1501,50 +1498,50 @@
         <v>1</v>
       </c>
       <c r="B28" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="C28" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="D28" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="E28" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
     </row>
     <row r="29" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A29">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="B29" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="C29" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="D29" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="E29" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
     </row>
     <row r="30" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A30">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B30" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="C30" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="D30" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="E30" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
     </row>
     <row r="31" spans="1:5" x14ac:dyDescent="0.2">
@@ -1552,16 +1549,16 @@
         <v>1</v>
       </c>
       <c r="B31" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="C31" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="D31" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="E31" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
     </row>
     <row r="32" spans="1:5" x14ac:dyDescent="0.2">
@@ -1569,16 +1566,16 @@
         <v>1</v>
       </c>
       <c r="B32" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="C32" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="D32" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="E32" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
     </row>
     <row r="33" spans="1:6" x14ac:dyDescent="0.2">
@@ -1586,16 +1583,19 @@
         <v>1</v>
       </c>
       <c r="B33" t="s">
+        <v>126</v>
+      </c>
+      <c r="C33" t="s">
+        <v>123</v>
+      </c>
+      <c r="D33" t="s">
+        <v>124</v>
+      </c>
+      <c r="E33" t="s">
         <v>125</v>
       </c>
-      <c r="C33" t="s">
-        <v>126</v>
-      </c>
-      <c r="D33" t="s">
-        <v>127</v>
-      </c>
-      <c r="E33" t="s">
-        <v>128</v>
+      <c r="F33" t="s">
+        <v>5</v>
       </c>
     </row>
     <row r="34" spans="1:6" x14ac:dyDescent="0.2">
@@ -1603,19 +1603,16 @@
         <v>1</v>
       </c>
       <c r="B34" t="s">
+        <v>127</v>
+      </c>
+      <c r="C34" t="s">
+        <v>128</v>
+      </c>
+      <c r="D34" t="s">
         <v>129</v>
       </c>
-      <c r="C34" t="s">
-        <v>126</v>
-      </c>
-      <c r="D34" t="s">
-        <v>127</v>
-      </c>
       <c r="E34" t="s">
-        <v>128</v>
-      </c>
-      <c r="F34" t="s">
-        <v>5</v>
+        <v>130</v>
       </c>
     </row>
     <row r="35" spans="1:6" x14ac:dyDescent="0.2">
@@ -1623,16 +1620,16 @@
         <v>1</v>
       </c>
       <c r="B35" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="C35" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="D35" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="E35" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
     </row>
     <row r="36" spans="1:6" x14ac:dyDescent="0.2">
@@ -1640,50 +1637,50 @@
         <v>1</v>
       </c>
       <c r="B36" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="C36" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="D36" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="E36" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
     </row>
     <row r="37" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A37">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="B37" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="C37" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="D37" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="E37" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
     </row>
     <row r="38" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A38">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B38" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="C38" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="D38" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="E38" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
     </row>
     <row r="39" spans="1:6" x14ac:dyDescent="0.2">
@@ -1691,16 +1688,16 @@
         <v>1</v>
       </c>
       <c r="B39" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="C39" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="D39" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="E39" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
     </row>
     <row r="40" spans="1:6" x14ac:dyDescent="0.2">
@@ -1708,38 +1705,38 @@
         <v>1</v>
       </c>
       <c r="B40" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="C40" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="D40" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="E40" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
     </row>
     <row r="41" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A41">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="B41" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="C41" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="D41" t="s">
+        <v>157</v>
+      </c>
+      <c r="E41" t="s">
         <v>156</v>
-      </c>
-      <c r="E41" t="s">
-        <v>157</v>
       </c>
     </row>
     <row r="42" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A42">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B42" t="s">
         <v>158</v>
@@ -1747,22 +1744,22 @@
       <c r="C42" t="s">
         <v>159</v>
       </c>
-      <c r="D42" t="s">
-        <v>160</v>
-      </c>
-      <c r="E42" t="s">
-        <v>159</v>
-      </c>
     </row>
     <row r="43" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A43">
         <v>1</v>
       </c>
       <c r="B43" t="s">
+        <v>160</v>
+      </c>
+      <c r="C43" t="s">
         <v>161</v>
       </c>
+      <c r="D43" t="s">
+        <v>162</v>
+      </c>
       <c r="E43" t="s">
-        <v>202</v>
+        <v>161</v>
       </c>
     </row>
     <row r="44" spans="1:6" x14ac:dyDescent="0.2">
@@ -1770,16 +1767,16 @@
         <v>1</v>
       </c>
       <c r="B44" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="C44" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="D44" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="E44" t="s">
-        <v>163</v>
+        <v>166</v>
       </c>
     </row>
     <row r="45" spans="1:6" x14ac:dyDescent="0.2">
@@ -1787,13 +1784,13 @@
         <v>1</v>
       </c>
       <c r="B45" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="C45" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="D45" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
       <c r="E45" t="s">
         <v>168</v>
@@ -1804,16 +1801,16 @@
         <v>1</v>
       </c>
       <c r="B46" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="C46" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="D46" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="E46" t="s">
-        <v>170</v>
+        <v>173</v>
       </c>
     </row>
     <row r="47" spans="1:6" x14ac:dyDescent="0.2">
@@ -1821,16 +1818,16 @@
         <v>1</v>
       </c>
       <c r="B47" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
       <c r="C47" t="s">
-        <v>173</v>
+        <v>175</v>
       </c>
       <c r="D47" t="s">
-        <v>174</v>
+        <v>176</v>
       </c>
       <c r="E47" t="s">
-        <v>175</v>
+        <v>177</v>
       </c>
     </row>
     <row r="48" spans="1:6" x14ac:dyDescent="0.2">
@@ -1838,13 +1835,13 @@
         <v>1</v>
       </c>
       <c r="B48" t="s">
-        <v>176</v>
+        <v>178</v>
       </c>
       <c r="C48" t="s">
-        <v>177</v>
+        <v>179</v>
       </c>
       <c r="D48" t="s">
-        <v>178</v>
+        <v>180</v>
       </c>
       <c r="E48" t="s">
         <v>179</v>
@@ -1855,16 +1852,16 @@
         <v>1</v>
       </c>
       <c r="B49" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="C49" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="D49" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="E49" t="s">
-        <v>181</v>
+        <v>184</v>
       </c>
     </row>
     <row r="50" spans="1:5" x14ac:dyDescent="0.2">
@@ -1872,16 +1869,16 @@
         <v>1</v>
       </c>
       <c r="B50" t="s">
-        <v>183</v>
+        <v>185</v>
       </c>
       <c r="C50" t="s">
-        <v>184</v>
+        <v>186</v>
       </c>
       <c r="D50" t="s">
-        <v>185</v>
+        <v>187</v>
       </c>
       <c r="E50" t="s">
-        <v>186</v>
+        <v>188</v>
       </c>
     </row>
     <row r="51" spans="1:5" x14ac:dyDescent="0.2">
@@ -1889,16 +1886,16 @@
         <v>1</v>
       </c>
       <c r="B51" t="s">
-        <v>187</v>
+        <v>189</v>
       </c>
       <c r="C51" t="s">
-        <v>188</v>
+        <v>190</v>
       </c>
       <c r="D51" t="s">
-        <v>189</v>
+        <v>191</v>
       </c>
       <c r="E51" t="s">
-        <v>190</v>
+        <v>192</v>
       </c>
     </row>
     <row r="52" spans="1:5" x14ac:dyDescent="0.2">
@@ -1906,16 +1903,13 @@
         <v>1</v>
       </c>
       <c r="B52" t="s">
-        <v>191</v>
+        <v>193</v>
       </c>
       <c r="C52" t="s">
-        <v>192</v>
-      </c>
-      <c r="D52" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="E52" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
     </row>
     <row r="53" spans="1:5" x14ac:dyDescent="0.2">
@@ -1923,13 +1917,16 @@
         <v>1</v>
       </c>
       <c r="B53" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="C53" t="s">
-        <v>196</v>
+        <v>197</v>
+      </c>
+      <c r="D53" t="s">
+        <v>198</v>
       </c>
       <c r="E53" t="s">
-        <v>197</v>
+        <v>199</v>
       </c>
     </row>
     <row r="54" spans="1:5" x14ac:dyDescent="0.2">
@@ -1937,16 +1934,16 @@
         <v>1</v>
       </c>
       <c r="B54" t="s">
-        <v>198</v>
+        <v>200</v>
       </c>
       <c r="C54" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
       <c r="D54" t="s">
-        <v>200</v>
+        <v>202</v>
       </c>
       <c r="E54" t="s">
-        <v>201</v>
+        <v>203</v>
       </c>
     </row>
   </sheetData>
@@ -1960,577 +1957,576 @@
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="5.6640625" customWidth="1"/>
-    <col min="2" max="2" width="30.6640625" style="3" customWidth="1"/>
-    <col min="3" max="4" width="30.6640625" customWidth="1"/>
+    <col min="2" max="4" width="30.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" ht="16" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="2" t="s">
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" ht="32" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A2">
         <v>15</v>
       </c>
-      <c r="B2" s="3" t="s">
+      <c r="B2" t="s">
         <v>6</v>
       </c>
       <c r="C2" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="3" spans="1:3" ht="16" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A3">
         <v>1</v>
       </c>
-      <c r="B3" s="3" t="s">
+      <c r="B3" t="s">
         <v>10</v>
       </c>
       <c r="C3" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="4" spans="1:3" ht="32" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A4">
-        <v>10</v>
-      </c>
-      <c r="B4" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="B4" t="s">
         <v>14</v>
       </c>
       <c r="C4" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="5" spans="1:3" ht="16" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A5">
-        <v>1</v>
-      </c>
-      <c r="B5" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="B5" t="s">
         <v>18</v>
       </c>
       <c r="C5" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="6" spans="1:3" ht="16" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A6">
-        <v>2</v>
-      </c>
-      <c r="B6" s="3" t="s">
+        <v>1</v>
+      </c>
+      <c r="B6" t="s">
         <v>22</v>
       </c>
       <c r="C6" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="7" spans="1:3" ht="16" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A7">
-        <v>1</v>
-      </c>
-      <c r="B7" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="B7" t="s">
         <v>26</v>
       </c>
       <c r="C7" t="s">
         <v>28</v>
       </c>
     </row>
-    <row r="8" spans="1:3" ht="16" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A8">
-        <v>3</v>
-      </c>
-      <c r="B8" s="3" t="s">
+        <v>1</v>
+      </c>
+      <c r="B8" t="s">
         <v>30</v>
       </c>
       <c r="C8" t="s">
         <v>32</v>
       </c>
     </row>
-    <row r="9" spans="1:3" ht="16" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A9">
-        <v>1</v>
-      </c>
-      <c r="B9" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="B9" t="s">
         <v>34</v>
       </c>
       <c r="C9" t="s">
         <v>36</v>
       </c>
     </row>
-    <row r="10" spans="1:3" ht="16" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A10">
-        <v>2</v>
-      </c>
-      <c r="B10" s="3" t="s">
+        <v>1</v>
+      </c>
+      <c r="B10" t="s">
         <v>38</v>
       </c>
       <c r="C10" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="11" spans="1:3" ht="16" x14ac:dyDescent="0.2">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A11">
         <v>2</v>
       </c>
-      <c r="B11" s="3" t="s">
-        <v>41</v>
+      <c r="B11" t="s">
+        <v>42</v>
       </c>
       <c r="C11" t="s">
         <v>43</v>
       </c>
     </row>
-    <row r="12" spans="1:3" ht="16" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A12">
-        <v>1</v>
-      </c>
-      <c r="B12" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="B12" t="s">
         <v>45</v>
       </c>
       <c r="C12" t="s">
         <v>47</v>
       </c>
     </row>
-    <row r="13" spans="1:3" ht="16" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A13">
         <v>1</v>
       </c>
-      <c r="B13" s="3" t="s">
+      <c r="B13" t="s">
         <v>49</v>
       </c>
       <c r="C13" t="s">
         <v>51</v>
       </c>
     </row>
-    <row r="14" spans="1:3" ht="16" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A14">
         <v>1</v>
       </c>
-      <c r="B14" s="3" t="s">
+      <c r="B14" t="s">
         <v>53</v>
       </c>
       <c r="C14" t="s">
         <v>55</v>
       </c>
     </row>
-    <row r="15" spans="1:3" ht="16" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A15">
         <v>1</v>
       </c>
-      <c r="B15" s="3" t="s">
+      <c r="B15" t="s">
         <v>57</v>
       </c>
       <c r="C15" t="s">
         <v>59</v>
       </c>
     </row>
-    <row r="16" spans="1:3" ht="16" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A16">
         <v>1</v>
       </c>
-      <c r="B16" s="3" t="s">
+      <c r="B16" t="s">
         <v>61</v>
       </c>
       <c r="C16" t="s">
         <v>63</v>
       </c>
     </row>
-    <row r="17" spans="1:3" ht="16" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A17">
         <v>1</v>
       </c>
-      <c r="B17" s="3" t="s">
+      <c r="B17" t="s">
         <v>65</v>
       </c>
       <c r="C17" t="s">
         <v>67</v>
       </c>
     </row>
-    <row r="18" spans="1:3" ht="16" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A18">
         <v>1</v>
       </c>
-      <c r="B18" s="3" t="s">
+      <c r="B18" t="s">
         <v>69</v>
       </c>
       <c r="C18" t="s">
         <v>71</v>
       </c>
     </row>
-    <row r="19" spans="1:3" ht="16" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A19">
         <v>1</v>
       </c>
-      <c r="B19" s="3" t="s">
+      <c r="B19" t="s">
         <v>72</v>
       </c>
       <c r="C19" t="s">
         <v>74</v>
       </c>
     </row>
-    <row r="20" spans="1:3" ht="16" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A20">
         <v>1</v>
       </c>
-      <c r="B20" s="3" t="s">
+      <c r="B20" t="s">
         <v>76</v>
       </c>
       <c r="C20" t="s">
         <v>78</v>
       </c>
     </row>
-    <row r="21" spans="1:3" ht="16" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A21">
         <v>1</v>
       </c>
-      <c r="B21" s="3" t="s">
+      <c r="B21" t="s">
         <v>79</v>
       </c>
       <c r="C21" t="s">
         <v>81</v>
       </c>
     </row>
-    <row r="22" spans="1:3" ht="16" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A22">
         <v>1</v>
       </c>
-      <c r="B22" s="3" t="s">
+      <c r="B22" t="s">
         <v>83</v>
       </c>
       <c r="C22" t="s">
         <v>85</v>
       </c>
     </row>
-    <row r="23" spans="1:3" ht="16" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A23">
-        <v>1</v>
-      </c>
-      <c r="B23" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="B23" t="s">
         <v>87</v>
       </c>
       <c r="C23" t="s">
         <v>89</v>
       </c>
     </row>
-    <row r="24" spans="1:3" ht="16" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A24">
-        <v>1</v>
-      </c>
-      <c r="B24" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="B24" t="s">
         <v>90</v>
       </c>
       <c r="C24" t="s">
         <v>92</v>
       </c>
     </row>
-    <row r="25" spans="1:3" ht="16" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A25">
-        <v>6</v>
-      </c>
-      <c r="B25" s="3" t="s">
-        <v>93</v>
+        <v>2</v>
+      </c>
+      <c r="B25" t="s">
+        <v>94</v>
       </c>
       <c r="C25" t="s">
-        <v>95</v>
-      </c>
-    </row>
-    <row r="26" spans="1:3" ht="16" x14ac:dyDescent="0.2">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="26" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A26">
+        <v>1</v>
+      </c>
+      <c r="B26" t="s">
+        <v>98</v>
+      </c>
+      <c r="C26" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="27" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A27">
+        <v>1</v>
+      </c>
+      <c r="B27" t="s">
+        <v>102</v>
+      </c>
+      <c r="C27" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="28" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A28">
+        <v>1</v>
+      </c>
+      <c r="B28" t="s">
+        <v>106</v>
+      </c>
+      <c r="C28" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="29" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A29">
         <v>2</v>
       </c>
-      <c r="B26" s="3" t="s">
-        <v>97</v>
-      </c>
-      <c r="C26" t="s">
-        <v>99</v>
-      </c>
-    </row>
-    <row r="27" spans="1:3" ht="16" x14ac:dyDescent="0.2">
-      <c r="A27">
-        <v>1</v>
-      </c>
-      <c r="B27" s="3" t="s">
-        <v>101</v>
-      </c>
-      <c r="C27" t="s">
-        <v>103</v>
-      </c>
-    </row>
-    <row r="28" spans="1:3" ht="16" x14ac:dyDescent="0.2">
-      <c r="A28">
-        <v>1</v>
-      </c>
-      <c r="B28" s="3" t="s">
-        <v>105</v>
-      </c>
-      <c r="C28" t="s">
-        <v>107</v>
-      </c>
-    </row>
-    <row r="29" spans="1:3" ht="16" x14ac:dyDescent="0.2">
-      <c r="A29">
-        <v>1</v>
-      </c>
-      <c r="B29" s="3" t="s">
-        <v>109</v>
+      <c r="B29" t="s">
+        <v>110</v>
       </c>
       <c r="C29" t="s">
-        <v>111</v>
-      </c>
-    </row>
-    <row r="30" spans="1:3" ht="16" x14ac:dyDescent="0.2">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="30" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A30">
+        <v>1</v>
+      </c>
+      <c r="B30" t="s">
+        <v>114</v>
+      </c>
+      <c r="C30" t="s">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="31" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A31">
+        <v>1</v>
+      </c>
+      <c r="B31" t="s">
+        <v>118</v>
+      </c>
+      <c r="C31" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="32" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A32">
+        <v>1</v>
+      </c>
+      <c r="B32" t="s">
+        <v>122</v>
+      </c>
+      <c r="C32" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="33" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A33">
+        <v>1</v>
+      </c>
+      <c r="B33" t="s">
+        <v>127</v>
+      </c>
+      <c r="C33" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="34" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A34">
+        <v>1</v>
+      </c>
+      <c r="B34" t="s">
+        <v>131</v>
+      </c>
+      <c r="C34" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="35" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A35">
+        <v>1</v>
+      </c>
+      <c r="B35" t="s">
+        <v>135</v>
+      </c>
+      <c r="C35" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="36" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A36">
         <v>2</v>
       </c>
-      <c r="B30" s="3" t="s">
-        <v>113</v>
-      </c>
-      <c r="C30" t="s">
-        <v>115</v>
-      </c>
-    </row>
-    <row r="31" spans="1:3" ht="16" x14ac:dyDescent="0.2">
-      <c r="A31">
-        <v>1</v>
-      </c>
-      <c r="B31" s="3" t="s">
-        <v>117</v>
-      </c>
-      <c r="C31" t="s">
-        <v>119</v>
-      </c>
-    </row>
-    <row r="32" spans="1:3" ht="16" x14ac:dyDescent="0.2">
-      <c r="A32">
-        <v>1</v>
-      </c>
-      <c r="B32" s="3" t="s">
-        <v>121</v>
-      </c>
-      <c r="C32" t="s">
-        <v>123</v>
-      </c>
-    </row>
-    <row r="33" spans="1:3" ht="16" x14ac:dyDescent="0.2">
-      <c r="A33">
-        <v>1</v>
-      </c>
-      <c r="B33" s="3" t="s">
-        <v>125</v>
-      </c>
-      <c r="C33" t="s">
-        <v>127</v>
-      </c>
-    </row>
-    <row r="34" spans="1:3" ht="16" x14ac:dyDescent="0.2">
-      <c r="A34">
-        <v>1</v>
-      </c>
-      <c r="B34" s="3" t="s">
-        <v>130</v>
-      </c>
-      <c r="C34" t="s">
-        <v>132</v>
-      </c>
-    </row>
-    <row r="35" spans="1:3" ht="16" x14ac:dyDescent="0.2">
-      <c r="A35">
-        <v>1</v>
-      </c>
-      <c r="B35" s="3" t="s">
-        <v>134</v>
-      </c>
-      <c r="C35" t="s">
-        <v>136</v>
-      </c>
-    </row>
-    <row r="36" spans="1:3" ht="16" x14ac:dyDescent="0.2">
-      <c r="A36">
-        <v>1</v>
-      </c>
-      <c r="B36" s="3" t="s">
-        <v>138</v>
+      <c r="B36" t="s">
+        <v>139</v>
       </c>
       <c r="C36" t="s">
-        <v>140</v>
-      </c>
-    </row>
-    <row r="37" spans="1:3" ht="16" x14ac:dyDescent="0.2">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="37" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A37">
+        <v>1</v>
+      </c>
+      <c r="B37" t="s">
+        <v>143</v>
+      </c>
+      <c r="C37" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="38" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A38">
+        <v>1</v>
+      </c>
+      <c r="B38" t="s">
+        <v>147</v>
+      </c>
+      <c r="C38" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="39" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A39">
+        <v>1</v>
+      </c>
+      <c r="B39" t="s">
+        <v>151</v>
+      </c>
+      <c r="C39" t="s">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="40" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A40">
         <v>2</v>
       </c>
-      <c r="B37" s="3" t="s">
-        <v>142</v>
-      </c>
-      <c r="C37" t="s">
-        <v>144</v>
-      </c>
-    </row>
-    <row r="38" spans="1:3" ht="16" x14ac:dyDescent="0.2">
-      <c r="A38">
-        <v>1</v>
-      </c>
-      <c r="B38" s="3" t="s">
-        <v>146</v>
-      </c>
-      <c r="C38" t="s">
-        <v>148</v>
-      </c>
-    </row>
-    <row r="39" spans="1:3" ht="16" x14ac:dyDescent="0.2">
-      <c r="A39">
-        <v>1</v>
-      </c>
-      <c r="B39" s="3" t="s">
-        <v>150</v>
-      </c>
-      <c r="C39" t="s">
-        <v>152</v>
-      </c>
-    </row>
-    <row r="40" spans="1:3" ht="16" x14ac:dyDescent="0.2">
-      <c r="A40">
-        <v>1</v>
-      </c>
-      <c r="B40" s="3" t="s">
-        <v>154</v>
+      <c r="B40" t="s">
+        <v>155</v>
       </c>
       <c r="C40" t="s">
-        <v>156</v>
-      </c>
-    </row>
-    <row r="41" spans="1:3" ht="16" x14ac:dyDescent="0.2">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="41" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A41">
-        <v>2</v>
-      </c>
-      <c r="B41" s="3" t="s">
-        <v>158</v>
+        <v>1</v>
+      </c>
+      <c r="B41" t="s">
+        <v>160</v>
       </c>
       <c r="C41" t="s">
-        <v>160</v>
-      </c>
-    </row>
-    <row r="42" spans="1:3" ht="16" x14ac:dyDescent="0.2">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="42" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A42">
         <v>1</v>
       </c>
-      <c r="B42" s="3" t="s">
-        <v>162</v>
+      <c r="B42" t="s">
+        <v>163</v>
       </c>
       <c r="C42" t="s">
-        <v>164</v>
-      </c>
-    </row>
-    <row r="43" spans="1:3" ht="16" x14ac:dyDescent="0.2">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="43" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A43">
         <v>1</v>
       </c>
-      <c r="B43" s="3" t="s">
-        <v>165</v>
+      <c r="B43" t="s">
+        <v>167</v>
       </c>
       <c r="C43" t="s">
-        <v>167</v>
-      </c>
-    </row>
-    <row r="44" spans="1:3" ht="16" x14ac:dyDescent="0.2">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="44" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A44">
         <v>1</v>
       </c>
-      <c r="B44" s="3" t="s">
-        <v>169</v>
+      <c r="B44" t="s">
+        <v>170</v>
       </c>
       <c r="C44" t="s">
-        <v>171</v>
-      </c>
-    </row>
-    <row r="45" spans="1:3" ht="16" x14ac:dyDescent="0.2">
+        <v>172</v>
+      </c>
+    </row>
+    <row r="45" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A45">
         <v>1</v>
       </c>
-      <c r="B45" s="3" t="s">
-        <v>172</v>
+      <c r="B45" t="s">
+        <v>174</v>
       </c>
       <c r="C45" t="s">
-        <v>174</v>
-      </c>
-    </row>
-    <row r="46" spans="1:3" ht="16" x14ac:dyDescent="0.2">
+        <v>176</v>
+      </c>
+    </row>
+    <row r="46" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A46">
         <v>1</v>
       </c>
-      <c r="B46" s="3" t="s">
-        <v>176</v>
+      <c r="B46" t="s">
+        <v>178</v>
       </c>
       <c r="C46" t="s">
-        <v>178</v>
-      </c>
-    </row>
-    <row r="47" spans="1:3" ht="16" x14ac:dyDescent="0.2">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="47" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A47">
         <v>1</v>
       </c>
-      <c r="B47" s="3" t="s">
-        <v>180</v>
+      <c r="B47" t="s">
+        <v>181</v>
       </c>
       <c r="C47" t="s">
-        <v>182</v>
-      </c>
-    </row>
-    <row r="48" spans="1:3" ht="16" x14ac:dyDescent="0.2">
+        <v>183</v>
+      </c>
+    </row>
+    <row r="48" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A48">
         <v>1</v>
       </c>
-      <c r="B48" s="3" t="s">
-        <v>183</v>
+      <c r="B48" t="s">
+        <v>185</v>
       </c>
       <c r="C48" t="s">
-        <v>185</v>
-      </c>
-    </row>
-    <row r="49" spans="1:3" ht="16" x14ac:dyDescent="0.2">
+        <v>187</v>
+      </c>
+    </row>
+    <row r="49" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A49">
         <v>1</v>
       </c>
-      <c r="B49" s="3" t="s">
-        <v>187</v>
+      <c r="B49" t="s">
+        <v>189</v>
       </c>
       <c r="C49" t="s">
-        <v>189</v>
-      </c>
-    </row>
-    <row r="50" spans="1:3" ht="16" x14ac:dyDescent="0.2">
+        <v>191</v>
+      </c>
+    </row>
+    <row r="50" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A50">
         <v>1</v>
       </c>
-      <c r="B50" s="3" t="s">
-        <v>191</v>
-      </c>
-      <c r="C50" t="s">
+      <c r="B50" t="s">
         <v>193</v>
       </c>
     </row>
-    <row r="51" spans="1:3" ht="16" x14ac:dyDescent="0.2">
+    <row r="51" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A51">
         <v>1</v>
       </c>
-      <c r="B51" s="3" t="s">
-        <v>195</v>
-      </c>
-    </row>
-    <row r="52" spans="1:3" ht="16" x14ac:dyDescent="0.2">
+      <c r="B51" t="s">
+        <v>196</v>
+      </c>
+      <c r="C51" t="s">
+        <v>198</v>
+      </c>
+    </row>
+    <row r="52" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A52">
         <v>1</v>
       </c>
-      <c r="B52" s="3" t="s">
-        <v>198</v>
+      <c r="B52" t="s">
+        <v>200</v>
       </c>
       <c r="C52" t="s">
-        <v>200</v>
+        <v>202</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
generated gerbers, updated BOM C18 error
</commit_message>
<xml_diff>
--- a/manufacturing files/blockaxe1 BOM.xlsx
+++ b/manufacturing files/blockaxe1 BOM.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/skot/Work/Bitcoin/blockaxe/blockaxe1/manufacturing files/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{29FC904F-6887-2E44-8DD1-926F5CC7C9A9}" xr6:coauthVersionLast="46" xr6:coauthVersionMax="46" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D38E2057-84C0-3C49-AEEB-D3FA35CF3D6D}" xr6:coauthVersionLast="46" xr6:coauthVersionMax="46" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="240" yWindow="500" windowWidth="28500" windowHeight="25000" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="240" yWindow="500" windowWidth="28500" windowHeight="25000" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="BOM" sheetId="1" r:id="rId1"/>
@@ -95,9 +95,6 @@
     <t>10uF</t>
   </si>
   <si>
-    <t>399-C0805C106K8PAC7800DKR-ND</t>
-  </si>
-  <si>
     <t>C0805C106K8PAC7800</t>
   </si>
   <si>
@@ -633,6 +630,9 @@
   </si>
   <si>
     <t>ECS-80-12-33-JGN-TR</t>
+  </si>
+  <si>
+    <t>399-C0805C106K8PAC7800CT-ND</t>
   </si>
 </sst>
 </file>
@@ -1130,10 +1130,10 @@
         <v>23</v>
       </c>
       <c r="D6" t="s">
+        <v>203</v>
+      </c>
+      <c r="E6" t="s">
         <v>24</v>
-      </c>
-      <c r="E6" t="s">
-        <v>25</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.2">
@@ -1141,16 +1141,16 @@
         <v>2</v>
       </c>
       <c r="B7" t="s">
+        <v>25</v>
+      </c>
+      <c r="C7" t="s">
         <v>26</v>
       </c>
-      <c r="C7" t="s">
+      <c r="D7" t="s">
         <v>27</v>
       </c>
-      <c r="D7" t="s">
+      <c r="E7" t="s">
         <v>28</v>
-      </c>
-      <c r="E7" t="s">
-        <v>29</v>
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.2">
@@ -1158,16 +1158,16 @@
         <v>1</v>
       </c>
       <c r="B8" t="s">
+        <v>29</v>
+      </c>
+      <c r="C8" t="s">
         <v>30</v>
       </c>
-      <c r="C8" t="s">
+      <c r="D8" t="s">
         <v>31</v>
       </c>
-      <c r="D8" t="s">
+      <c r="E8" t="s">
         <v>32</v>
-      </c>
-      <c r="E8" t="s">
-        <v>33</v>
       </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.2">
@@ -1175,16 +1175,16 @@
         <v>3</v>
       </c>
       <c r="B9" t="s">
+        <v>33</v>
+      </c>
+      <c r="C9" t="s">
         <v>34</v>
       </c>
-      <c r="C9" t="s">
+      <c r="D9" t="s">
         <v>35</v>
       </c>
-      <c r="D9" t="s">
+      <c r="E9" t="s">
         <v>36</v>
-      </c>
-      <c r="E9" t="s">
-        <v>37</v>
       </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.2">
@@ -1192,16 +1192,16 @@
         <v>1</v>
       </c>
       <c r="B10" t="s">
+        <v>37</v>
+      </c>
+      <c r="C10" t="s">
         <v>38</v>
       </c>
-      <c r="C10" t="s">
+      <c r="D10" t="s">
         <v>39</v>
       </c>
-      <c r="D10" t="s">
+      <c r="E10" t="s">
         <v>40</v>
-      </c>
-      <c r="E10" t="s">
-        <v>41</v>
       </c>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.2">
@@ -1209,16 +1209,16 @@
         <v>2</v>
       </c>
       <c r="B11" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C11" t="s">
         <v>19</v>
       </c>
       <c r="D11" t="s">
+        <v>42</v>
+      </c>
+      <c r="E11" t="s">
         <v>43</v>
-      </c>
-      <c r="E11" t="s">
-        <v>44</v>
       </c>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.2">
@@ -1226,16 +1226,16 @@
         <v>2</v>
       </c>
       <c r="B12" t="s">
+        <v>44</v>
+      </c>
+      <c r="C12" t="s">
         <v>45</v>
       </c>
-      <c r="C12" t="s">
+      <c r="D12" t="s">
         <v>46</v>
       </c>
-      <c r="D12" t="s">
+      <c r="E12" t="s">
         <v>47</v>
-      </c>
-      <c r="E12" t="s">
-        <v>48</v>
       </c>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.2">
@@ -1243,16 +1243,16 @@
         <v>1</v>
       </c>
       <c r="B13" t="s">
+        <v>48</v>
+      </c>
+      <c r="C13" t="s">
         <v>49</v>
       </c>
-      <c r="C13" t="s">
+      <c r="D13" t="s">
         <v>50</v>
       </c>
-      <c r="D13" t="s">
+      <c r="E13" t="s">
         <v>51</v>
-      </c>
-      <c r="E13" t="s">
-        <v>52</v>
       </c>
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.2">
@@ -1260,16 +1260,16 @@
         <v>1</v>
       </c>
       <c r="B14" t="s">
+        <v>52</v>
+      </c>
+      <c r="C14" t="s">
         <v>53</v>
       </c>
-      <c r="C14" t="s">
+      <c r="D14" t="s">
         <v>54</v>
       </c>
-      <c r="D14" t="s">
+      <c r="E14" t="s">
         <v>55</v>
-      </c>
-      <c r="E14" t="s">
-        <v>56</v>
       </c>
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.2">
@@ -1277,16 +1277,16 @@
         <v>1</v>
       </c>
       <c r="B15" t="s">
+        <v>56</v>
+      </c>
+      <c r="C15" t="s">
         <v>57</v>
       </c>
-      <c r="C15" t="s">
+      <c r="D15" t="s">
         <v>58</v>
       </c>
-      <c r="D15" t="s">
+      <c r="E15" t="s">
         <v>59</v>
-      </c>
-      <c r="E15" t="s">
-        <v>60</v>
       </c>
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.2">
@@ -1294,16 +1294,16 @@
         <v>1</v>
       </c>
       <c r="B16" t="s">
+        <v>60</v>
+      </c>
+      <c r="C16" t="s">
         <v>61</v>
       </c>
-      <c r="C16" t="s">
+      <c r="D16" t="s">
         <v>62</v>
       </c>
-      <c r="D16" t="s">
+      <c r="E16" t="s">
         <v>63</v>
-      </c>
-      <c r="E16" t="s">
-        <v>64</v>
       </c>
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.2">
@@ -1311,16 +1311,16 @@
         <v>1</v>
       </c>
       <c r="B17" t="s">
+        <v>64</v>
+      </c>
+      <c r="C17" t="s">
         <v>65</v>
       </c>
-      <c r="C17" t="s">
+      <c r="D17" t="s">
         <v>66</v>
       </c>
-      <c r="D17" t="s">
+      <c r="E17" t="s">
         <v>67</v>
-      </c>
-      <c r="E17" t="s">
-        <v>68</v>
       </c>
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.2">
@@ -1328,16 +1328,16 @@
         <v>1</v>
       </c>
       <c r="B18" t="s">
+        <v>68</v>
+      </c>
+      <c r="C18" t="s">
         <v>69</v>
       </c>
-      <c r="C18" t="s">
+      <c r="D18" t="s">
         <v>70</v>
       </c>
-      <c r="D18" t="s">
-        <v>71</v>
-      </c>
       <c r="E18" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.2">
@@ -1345,16 +1345,16 @@
         <v>1</v>
       </c>
       <c r="B19" t="s">
+        <v>71</v>
+      </c>
+      <c r="C19" t="s">
         <v>72</v>
       </c>
-      <c r="C19" t="s">
+      <c r="D19" t="s">
         <v>73</v>
       </c>
-      <c r="D19" t="s">
+      <c r="E19" t="s">
         <v>74</v>
-      </c>
-      <c r="E19" t="s">
-        <v>75</v>
       </c>
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.2">
@@ -1362,16 +1362,16 @@
         <v>1</v>
       </c>
       <c r="B20" t="s">
+        <v>75</v>
+      </c>
+      <c r="C20" t="s">
         <v>76</v>
       </c>
-      <c r="C20" t="s">
+      <c r="D20" t="s">
         <v>77</v>
       </c>
-      <c r="D20" t="s">
-        <v>78</v>
-      </c>
       <c r="E20" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
     </row>
     <row r="21" spans="1:5" x14ac:dyDescent="0.2">
@@ -1379,16 +1379,16 @@
         <v>1</v>
       </c>
       <c r="B21" t="s">
+        <v>78</v>
+      </c>
+      <c r="C21" t="s">
         <v>79</v>
       </c>
-      <c r="C21" t="s">
+      <c r="D21" t="s">
         <v>80</v>
       </c>
-      <c r="D21" t="s">
+      <c r="E21" t="s">
         <v>81</v>
-      </c>
-      <c r="E21" t="s">
-        <v>82</v>
       </c>
     </row>
     <row r="22" spans="1:5" x14ac:dyDescent="0.2">
@@ -1396,16 +1396,16 @@
         <v>1</v>
       </c>
       <c r="B22" t="s">
+        <v>82</v>
+      </c>
+      <c r="C22" t="s">
         <v>83</v>
       </c>
-      <c r="C22" t="s">
+      <c r="D22" t="s">
         <v>84</v>
       </c>
-      <c r="D22" t="s">
+      <c r="E22" t="s">
         <v>85</v>
-      </c>
-      <c r="E22" t="s">
-        <v>86</v>
       </c>
     </row>
     <row r="23" spans="1:5" x14ac:dyDescent="0.2">
@@ -1413,16 +1413,16 @@
         <v>2</v>
       </c>
       <c r="B23" t="s">
+        <v>86</v>
+      </c>
+      <c r="C23" t="s">
         <v>87</v>
       </c>
-      <c r="C23" t="s">
+      <c r="D23" t="s">
         <v>88</v>
       </c>
-      <c r="D23" t="s">
-        <v>89</v>
-      </c>
       <c r="E23" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
     </row>
     <row r="24" spans="1:5" x14ac:dyDescent="0.2">
@@ -1430,16 +1430,16 @@
         <v>6</v>
       </c>
       <c r="B24" t="s">
+        <v>89</v>
+      </c>
+      <c r="C24" t="s">
         <v>90</v>
       </c>
-      <c r="C24" t="s">
+      <c r="D24" t="s">
         <v>91</v>
       </c>
-      <c r="D24" t="s">
+      <c r="E24" t="s">
         <v>92</v>
-      </c>
-      <c r="E24" t="s">
-        <v>93</v>
       </c>
     </row>
     <row r="25" spans="1:5" x14ac:dyDescent="0.2">
@@ -1447,16 +1447,16 @@
         <v>2</v>
       </c>
       <c r="B25" t="s">
+        <v>93</v>
+      </c>
+      <c r="C25" t="s">
         <v>94</v>
       </c>
-      <c r="C25" t="s">
+      <c r="D25" t="s">
         <v>95</v>
       </c>
-      <c r="D25" t="s">
+      <c r="E25" t="s">
         <v>96</v>
-      </c>
-      <c r="E25" t="s">
-        <v>97</v>
       </c>
     </row>
     <row r="26" spans="1:5" x14ac:dyDescent="0.2">
@@ -1464,16 +1464,16 @@
         <v>1</v>
       </c>
       <c r="B26" t="s">
+        <v>97</v>
+      </c>
+      <c r="C26" t="s">
         <v>98</v>
       </c>
-      <c r="C26" t="s">
+      <c r="D26" t="s">
         <v>99</v>
       </c>
-      <c r="D26" t="s">
+      <c r="E26" t="s">
         <v>100</v>
-      </c>
-      <c r="E26" t="s">
-        <v>101</v>
       </c>
     </row>
     <row r="27" spans="1:5" x14ac:dyDescent="0.2">
@@ -1481,16 +1481,16 @@
         <v>1</v>
       </c>
       <c r="B27" t="s">
+        <v>101</v>
+      </c>
+      <c r="C27" t="s">
         <v>102</v>
       </c>
-      <c r="C27" t="s">
+      <c r="D27" t="s">
         <v>103</v>
       </c>
-      <c r="D27" t="s">
+      <c r="E27" t="s">
         <v>104</v>
-      </c>
-      <c r="E27" t="s">
-        <v>105</v>
       </c>
     </row>
     <row r="28" spans="1:5" x14ac:dyDescent="0.2">
@@ -1498,16 +1498,16 @@
         <v>1</v>
       </c>
       <c r="B28" t="s">
+        <v>105</v>
+      </c>
+      <c r="C28" t="s">
         <v>106</v>
       </c>
-      <c r="C28" t="s">
+      <c r="D28" t="s">
         <v>107</v>
       </c>
-      <c r="D28" t="s">
+      <c r="E28" t="s">
         <v>108</v>
-      </c>
-      <c r="E28" t="s">
-        <v>109</v>
       </c>
     </row>
     <row r="29" spans="1:5" x14ac:dyDescent="0.2">
@@ -1515,16 +1515,16 @@
         <v>2</v>
       </c>
       <c r="B29" t="s">
+        <v>109</v>
+      </c>
+      <c r="C29" t="s">
         <v>110</v>
       </c>
-      <c r="C29" t="s">
+      <c r="D29" t="s">
         <v>111</v>
       </c>
-      <c r="D29" t="s">
+      <c r="E29" t="s">
         <v>112</v>
-      </c>
-      <c r="E29" t="s">
-        <v>113</v>
       </c>
     </row>
     <row r="30" spans="1:5" x14ac:dyDescent="0.2">
@@ -1532,16 +1532,16 @@
         <v>1</v>
       </c>
       <c r="B30" t="s">
+        <v>113</v>
+      </c>
+      <c r="C30" t="s">
         <v>114</v>
       </c>
-      <c r="C30" t="s">
+      <c r="D30" t="s">
         <v>115</v>
       </c>
-      <c r="D30" t="s">
+      <c r="E30" t="s">
         <v>116</v>
-      </c>
-      <c r="E30" t="s">
-        <v>117</v>
       </c>
     </row>
     <row r="31" spans="1:5" x14ac:dyDescent="0.2">
@@ -1549,16 +1549,16 @@
         <v>1</v>
       </c>
       <c r="B31" t="s">
+        <v>117</v>
+      </c>
+      <c r="C31" t="s">
         <v>118</v>
       </c>
-      <c r="C31" t="s">
+      <c r="D31" t="s">
         <v>119</v>
       </c>
-      <c r="D31" t="s">
+      <c r="E31" t="s">
         <v>120</v>
-      </c>
-      <c r="E31" t="s">
-        <v>121</v>
       </c>
     </row>
     <row r="32" spans="1:5" x14ac:dyDescent="0.2">
@@ -1566,16 +1566,16 @@
         <v>1</v>
       </c>
       <c r="B32" t="s">
+        <v>121</v>
+      </c>
+      <c r="C32" t="s">
         <v>122</v>
       </c>
-      <c r="C32" t="s">
+      <c r="D32" t="s">
         <v>123</v>
       </c>
-      <c r="D32" t="s">
+      <c r="E32" t="s">
         <v>124</v>
-      </c>
-      <c r="E32" t="s">
-        <v>125</v>
       </c>
     </row>
     <row r="33" spans="1:6" x14ac:dyDescent="0.2">
@@ -1583,16 +1583,16 @@
         <v>1</v>
       </c>
       <c r="B33" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="C33" t="s">
+        <v>122</v>
+      </c>
+      <c r="D33" t="s">
         <v>123</v>
       </c>
-      <c r="D33" t="s">
+      <c r="E33" t="s">
         <v>124</v>
-      </c>
-      <c r="E33" t="s">
-        <v>125</v>
       </c>
       <c r="F33" t="s">
         <v>5</v>
@@ -1603,16 +1603,16 @@
         <v>1</v>
       </c>
       <c r="B34" t="s">
+        <v>126</v>
+      </c>
+      <c r="C34" t="s">
         <v>127</v>
       </c>
-      <c r="C34" t="s">
+      <c r="D34" t="s">
         <v>128</v>
       </c>
-      <c r="D34" t="s">
+      <c r="E34" t="s">
         <v>129</v>
-      </c>
-      <c r="E34" t="s">
-        <v>130</v>
       </c>
     </row>
     <row r="35" spans="1:6" x14ac:dyDescent="0.2">
@@ -1620,16 +1620,16 @@
         <v>1</v>
       </c>
       <c r="B35" t="s">
+        <v>130</v>
+      </c>
+      <c r="C35" t="s">
         <v>131</v>
       </c>
-      <c r="C35" t="s">
+      <c r="D35" t="s">
         <v>132</v>
       </c>
-      <c r="D35" t="s">
+      <c r="E35" t="s">
         <v>133</v>
-      </c>
-      <c r="E35" t="s">
-        <v>134</v>
       </c>
     </row>
     <row r="36" spans="1:6" x14ac:dyDescent="0.2">
@@ -1637,16 +1637,16 @@
         <v>1</v>
       </c>
       <c r="B36" t="s">
+        <v>134</v>
+      </c>
+      <c r="C36" t="s">
         <v>135</v>
       </c>
-      <c r="C36" t="s">
+      <c r="D36" t="s">
         <v>136</v>
       </c>
-      <c r="D36" t="s">
+      <c r="E36" t="s">
         <v>137</v>
-      </c>
-      <c r="E36" t="s">
-        <v>138</v>
       </c>
     </row>
     <row r="37" spans="1:6" x14ac:dyDescent="0.2">
@@ -1654,16 +1654,16 @@
         <v>2</v>
       </c>
       <c r="B37" t="s">
+        <v>138</v>
+      </c>
+      <c r="C37" t="s">
         <v>139</v>
       </c>
-      <c r="C37" t="s">
+      <c r="D37" t="s">
         <v>140</v>
       </c>
-      <c r="D37" t="s">
+      <c r="E37" t="s">
         <v>141</v>
-      </c>
-      <c r="E37" t="s">
-        <v>142</v>
       </c>
     </row>
     <row r="38" spans="1:6" x14ac:dyDescent="0.2">
@@ -1671,16 +1671,16 @@
         <v>1</v>
       </c>
       <c r="B38" t="s">
+        <v>142</v>
+      </c>
+      <c r="C38" t="s">
         <v>143</v>
       </c>
-      <c r="C38" t="s">
+      <c r="D38" t="s">
         <v>144</v>
       </c>
-      <c r="D38" t="s">
+      <c r="E38" t="s">
         <v>145</v>
-      </c>
-      <c r="E38" t="s">
-        <v>146</v>
       </c>
     </row>
     <row r="39" spans="1:6" x14ac:dyDescent="0.2">
@@ -1688,16 +1688,16 @@
         <v>1</v>
       </c>
       <c r="B39" t="s">
+        <v>146</v>
+      </c>
+      <c r="C39" t="s">
         <v>147</v>
       </c>
-      <c r="C39" t="s">
+      <c r="D39" t="s">
         <v>148</v>
       </c>
-      <c r="D39" t="s">
+      <c r="E39" t="s">
         <v>149</v>
-      </c>
-      <c r="E39" t="s">
-        <v>150</v>
       </c>
     </row>
     <row r="40" spans="1:6" x14ac:dyDescent="0.2">
@@ -1705,16 +1705,16 @@
         <v>1</v>
       </c>
       <c r="B40" t="s">
+        <v>150</v>
+      </c>
+      <c r="C40" t="s">
         <v>151</v>
       </c>
-      <c r="C40" t="s">
+      <c r="D40" t="s">
         <v>152</v>
       </c>
-      <c r="D40" t="s">
+      <c r="E40" t="s">
         <v>153</v>
-      </c>
-      <c r="E40" t="s">
-        <v>154</v>
       </c>
     </row>
     <row r="41" spans="1:6" x14ac:dyDescent="0.2">
@@ -1722,16 +1722,16 @@
         <v>2</v>
       </c>
       <c r="B41" t="s">
+        <v>154</v>
+      </c>
+      <c r="C41" t="s">
         <v>155</v>
       </c>
-      <c r="C41" t="s">
+      <c r="D41" t="s">
         <v>156</v>
       </c>
-      <c r="D41" t="s">
-        <v>157</v>
-      </c>
       <c r="E41" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
     </row>
     <row r="42" spans="1:6" x14ac:dyDescent="0.2">
@@ -1739,10 +1739,10 @@
         <v>1</v>
       </c>
       <c r="B42" t="s">
+        <v>157</v>
+      </c>
+      <c r="C42" t="s">
         <v>158</v>
-      </c>
-      <c r="C42" t="s">
-        <v>159</v>
       </c>
     </row>
     <row r="43" spans="1:6" x14ac:dyDescent="0.2">
@@ -1750,16 +1750,16 @@
         <v>1</v>
       </c>
       <c r="B43" t="s">
+        <v>159</v>
+      </c>
+      <c r="C43" t="s">
         <v>160</v>
       </c>
-      <c r="C43" t="s">
+      <c r="D43" t="s">
         <v>161</v>
       </c>
-      <c r="D43" t="s">
-        <v>162</v>
-      </c>
       <c r="E43" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
     </row>
     <row r="44" spans="1:6" x14ac:dyDescent="0.2">
@@ -1767,16 +1767,16 @@
         <v>1</v>
       </c>
       <c r="B44" t="s">
+        <v>162</v>
+      </c>
+      <c r="C44" t="s">
         <v>163</v>
       </c>
-      <c r="C44" t="s">
+      <c r="D44" t="s">
         <v>164</v>
       </c>
-      <c r="D44" t="s">
+      <c r="E44" t="s">
         <v>165</v>
-      </c>
-      <c r="E44" t="s">
-        <v>166</v>
       </c>
     </row>
     <row r="45" spans="1:6" x14ac:dyDescent="0.2">
@@ -1784,16 +1784,16 @@
         <v>1</v>
       </c>
       <c r="B45" t="s">
+        <v>166</v>
+      </c>
+      <c r="C45" t="s">
         <v>167</v>
       </c>
-      <c r="C45" t="s">
+      <c r="D45" t="s">
         <v>168</v>
       </c>
-      <c r="D45" t="s">
-        <v>169</v>
-      </c>
       <c r="E45" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
     </row>
     <row r="46" spans="1:6" x14ac:dyDescent="0.2">
@@ -1801,16 +1801,16 @@
         <v>1</v>
       </c>
       <c r="B46" t="s">
+        <v>169</v>
+      </c>
+      <c r="C46" t="s">
         <v>170</v>
       </c>
-      <c r="C46" t="s">
+      <c r="D46" t="s">
         <v>171</v>
       </c>
-      <c r="D46" t="s">
+      <c r="E46" t="s">
         <v>172</v>
-      </c>
-      <c r="E46" t="s">
-        <v>173</v>
       </c>
     </row>
     <row r="47" spans="1:6" x14ac:dyDescent="0.2">
@@ -1818,16 +1818,16 @@
         <v>1</v>
       </c>
       <c r="B47" t="s">
+        <v>173</v>
+      </c>
+      <c r="C47" t="s">
         <v>174</v>
       </c>
-      <c r="C47" t="s">
+      <c r="D47" t="s">
         <v>175</v>
       </c>
-      <c r="D47" t="s">
+      <c r="E47" t="s">
         <v>176</v>
-      </c>
-      <c r="E47" t="s">
-        <v>177</v>
       </c>
     </row>
     <row r="48" spans="1:6" x14ac:dyDescent="0.2">
@@ -1835,16 +1835,16 @@
         <v>1</v>
       </c>
       <c r="B48" t="s">
+        <v>177</v>
+      </c>
+      <c r="C48" t="s">
         <v>178</v>
       </c>
-      <c r="C48" t="s">
+      <c r="D48" t="s">
         <v>179</v>
       </c>
-      <c r="D48" t="s">
-        <v>180</v>
-      </c>
       <c r="E48" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
     </row>
     <row r="49" spans="1:5" x14ac:dyDescent="0.2">
@@ -1852,16 +1852,16 @@
         <v>1</v>
       </c>
       <c r="B49" t="s">
+        <v>180</v>
+      </c>
+      <c r="C49" t="s">
         <v>181</v>
       </c>
-      <c r="C49" t="s">
+      <c r="D49" t="s">
         <v>182</v>
       </c>
-      <c r="D49" t="s">
+      <c r="E49" t="s">
         <v>183</v>
-      </c>
-      <c r="E49" t="s">
-        <v>184</v>
       </c>
     </row>
     <row r="50" spans="1:5" x14ac:dyDescent="0.2">
@@ -1869,16 +1869,16 @@
         <v>1</v>
       </c>
       <c r="B50" t="s">
+        <v>184</v>
+      </c>
+      <c r="C50" t="s">
         <v>185</v>
       </c>
-      <c r="C50" t="s">
+      <c r="D50" t="s">
         <v>186</v>
       </c>
-      <c r="D50" t="s">
+      <c r="E50" t="s">
         <v>187</v>
-      </c>
-      <c r="E50" t="s">
-        <v>188</v>
       </c>
     </row>
     <row r="51" spans="1:5" x14ac:dyDescent="0.2">
@@ -1886,16 +1886,16 @@
         <v>1</v>
       </c>
       <c r="B51" t="s">
+        <v>188</v>
+      </c>
+      <c r="C51" t="s">
         <v>189</v>
       </c>
-      <c r="C51" t="s">
+      <c r="D51" t="s">
         <v>190</v>
       </c>
-      <c r="D51" t="s">
+      <c r="E51" t="s">
         <v>191</v>
-      </c>
-      <c r="E51" t="s">
-        <v>192</v>
       </c>
     </row>
     <row r="52" spans="1:5" x14ac:dyDescent="0.2">
@@ -1903,13 +1903,13 @@
         <v>1</v>
       </c>
       <c r="B52" t="s">
+        <v>192</v>
+      </c>
+      <c r="C52" t="s">
         <v>193</v>
       </c>
-      <c r="C52" t="s">
+      <c r="E52" t="s">
         <v>194</v>
-      </c>
-      <c r="E52" t="s">
-        <v>195</v>
       </c>
     </row>
     <row r="53" spans="1:5" x14ac:dyDescent="0.2">
@@ -1917,16 +1917,16 @@
         <v>1</v>
       </c>
       <c r="B53" t="s">
+        <v>195</v>
+      </c>
+      <c r="C53" t="s">
         <v>196</v>
       </c>
-      <c r="C53" t="s">
+      <c r="D53" t="s">
         <v>197</v>
       </c>
-      <c r="D53" t="s">
+      <c r="E53" t="s">
         <v>198</v>
-      </c>
-      <c r="E53" t="s">
-        <v>199</v>
       </c>
     </row>
     <row r="54" spans="1:5" x14ac:dyDescent="0.2">
@@ -1934,16 +1934,16 @@
         <v>1</v>
       </c>
       <c r="B54" t="s">
+        <v>199</v>
+      </c>
+      <c r="C54" t="s">
         <v>200</v>
       </c>
-      <c r="C54" t="s">
+      <c r="D54" t="s">
         <v>201</v>
       </c>
-      <c r="D54" t="s">
+      <c r="E54" t="s">
         <v>202</v>
-      </c>
-      <c r="E54" t="s">
-        <v>203</v>
       </c>
     </row>
   </sheetData>
@@ -2023,7 +2023,7 @@
         <v>22</v>
       </c>
       <c r="C6" t="s">
-        <v>24</v>
+        <v>203</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.2">
@@ -2031,10 +2031,10 @@
         <v>2</v>
       </c>
       <c r="B7" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="C7" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.2">
@@ -2042,10 +2042,10 @@
         <v>1</v>
       </c>
       <c r="B8" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="C8" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.2">
@@ -2053,10 +2053,10 @@
         <v>3</v>
       </c>
       <c r="B9" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="C9" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.2">
@@ -2064,10 +2064,10 @@
         <v>1</v>
       </c>
       <c r="B10" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C10" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.2">
@@ -2075,10 +2075,10 @@
         <v>2</v>
       </c>
       <c r="B11" t="s">
+        <v>41</v>
+      </c>
+      <c r="C11" t="s">
         <v>42</v>
-      </c>
-      <c r="C11" t="s">
-        <v>43</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.2">
@@ -2086,10 +2086,10 @@
         <v>2</v>
       </c>
       <c r="B12" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="C12" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.2">
@@ -2097,10 +2097,10 @@
         <v>1</v>
       </c>
       <c r="B13" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="C13" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.2">
@@ -2108,10 +2108,10 @@
         <v>1</v>
       </c>
       <c r="B14" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="C14" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.2">
@@ -2119,10 +2119,10 @@
         <v>1</v>
       </c>
       <c r="B15" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="C15" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.2">
@@ -2130,10 +2130,10 @@
         <v>1</v>
       </c>
       <c r="B16" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="C16" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.2">
@@ -2141,10 +2141,10 @@
         <v>1</v>
       </c>
       <c r="B17" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="C17" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.2">
@@ -2152,10 +2152,10 @@
         <v>1</v>
       </c>
       <c r="B18" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="C18" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.2">
@@ -2163,10 +2163,10 @@
         <v>1</v>
       </c>
       <c r="B19" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="C19" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.2">
@@ -2174,10 +2174,10 @@
         <v>1</v>
       </c>
       <c r="B20" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="C20" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.2">
@@ -2185,10 +2185,10 @@
         <v>1</v>
       </c>
       <c r="B21" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="C21" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
     </row>
     <row r="22" spans="1:3" x14ac:dyDescent="0.2">
@@ -2196,10 +2196,10 @@
         <v>1</v>
       </c>
       <c r="B22" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="C22" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
     </row>
     <row r="23" spans="1:3" x14ac:dyDescent="0.2">
@@ -2207,10 +2207,10 @@
         <v>2</v>
       </c>
       <c r="B23" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="C23" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
     </row>
     <row r="24" spans="1:3" x14ac:dyDescent="0.2">
@@ -2218,10 +2218,10 @@
         <v>6</v>
       </c>
       <c r="B24" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="C24" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
     </row>
     <row r="25" spans="1:3" x14ac:dyDescent="0.2">
@@ -2229,10 +2229,10 @@
         <v>2</v>
       </c>
       <c r="B25" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="C25" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
     </row>
     <row r="26" spans="1:3" x14ac:dyDescent="0.2">
@@ -2240,10 +2240,10 @@
         <v>1</v>
       </c>
       <c r="B26" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="C26" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
     </row>
     <row r="27" spans="1:3" x14ac:dyDescent="0.2">
@@ -2251,10 +2251,10 @@
         <v>1</v>
       </c>
       <c r="B27" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="C27" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
     </row>
     <row r="28" spans="1:3" x14ac:dyDescent="0.2">
@@ -2262,10 +2262,10 @@
         <v>1</v>
       </c>
       <c r="B28" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="C28" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
     </row>
     <row r="29" spans="1:3" x14ac:dyDescent="0.2">
@@ -2273,10 +2273,10 @@
         <v>2</v>
       </c>
       <c r="B29" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="C29" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
     </row>
     <row r="30" spans="1:3" x14ac:dyDescent="0.2">
@@ -2284,10 +2284,10 @@
         <v>1</v>
       </c>
       <c r="B30" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="C30" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
     </row>
     <row r="31" spans="1:3" x14ac:dyDescent="0.2">
@@ -2295,10 +2295,10 @@
         <v>1</v>
       </c>
       <c r="B31" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="C31" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
     </row>
     <row r="32" spans="1:3" x14ac:dyDescent="0.2">
@@ -2306,10 +2306,10 @@
         <v>1</v>
       </c>
       <c r="B32" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="C32" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
     </row>
     <row r="33" spans="1:3" x14ac:dyDescent="0.2">
@@ -2317,10 +2317,10 @@
         <v>1</v>
       </c>
       <c r="B33" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="C33" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
     </row>
     <row r="34" spans="1:3" x14ac:dyDescent="0.2">
@@ -2328,10 +2328,10 @@
         <v>1</v>
       </c>
       <c r="B34" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="C34" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
     </row>
     <row r="35" spans="1:3" x14ac:dyDescent="0.2">
@@ -2339,10 +2339,10 @@
         <v>1</v>
       </c>
       <c r="B35" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="C35" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
     </row>
     <row r="36" spans="1:3" x14ac:dyDescent="0.2">
@@ -2350,10 +2350,10 @@
         <v>2</v>
       </c>
       <c r="B36" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="C36" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
     </row>
     <row r="37" spans="1:3" x14ac:dyDescent="0.2">
@@ -2361,10 +2361,10 @@
         <v>1</v>
       </c>
       <c r="B37" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="C37" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
     </row>
     <row r="38" spans="1:3" x14ac:dyDescent="0.2">
@@ -2372,10 +2372,10 @@
         <v>1</v>
       </c>
       <c r="B38" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="C38" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
     </row>
     <row r="39" spans="1:3" x14ac:dyDescent="0.2">
@@ -2383,10 +2383,10 @@
         <v>1</v>
       </c>
       <c r="B39" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="C39" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
     </row>
     <row r="40" spans="1:3" x14ac:dyDescent="0.2">
@@ -2394,10 +2394,10 @@
         <v>2</v>
       </c>
       <c r="B40" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="C40" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
     </row>
     <row r="41" spans="1:3" x14ac:dyDescent="0.2">
@@ -2405,10 +2405,10 @@
         <v>1</v>
       </c>
       <c r="B41" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="C41" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
     </row>
     <row r="42" spans="1:3" x14ac:dyDescent="0.2">
@@ -2416,10 +2416,10 @@
         <v>1</v>
       </c>
       <c r="B42" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="C42" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
     </row>
     <row r="43" spans="1:3" x14ac:dyDescent="0.2">
@@ -2427,10 +2427,10 @@
         <v>1</v>
       </c>
       <c r="B43" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="C43" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
     </row>
     <row r="44" spans="1:3" x14ac:dyDescent="0.2">
@@ -2438,10 +2438,10 @@
         <v>1</v>
       </c>
       <c r="B44" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="C44" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
     </row>
     <row r="45" spans="1:3" x14ac:dyDescent="0.2">
@@ -2449,10 +2449,10 @@
         <v>1</v>
       </c>
       <c r="B45" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="C45" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
     </row>
     <row r="46" spans="1:3" x14ac:dyDescent="0.2">
@@ -2460,10 +2460,10 @@
         <v>1</v>
       </c>
       <c r="B46" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="C46" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
     </row>
     <row r="47" spans="1:3" x14ac:dyDescent="0.2">
@@ -2471,10 +2471,10 @@
         <v>1</v>
       </c>
       <c r="B47" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="C47" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
     </row>
     <row r="48" spans="1:3" x14ac:dyDescent="0.2">
@@ -2482,10 +2482,10 @@
         <v>1</v>
       </c>
       <c r="B48" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="C48" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
     </row>
     <row r="49" spans="1:3" x14ac:dyDescent="0.2">
@@ -2493,10 +2493,10 @@
         <v>1</v>
       </c>
       <c r="B49" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="C49" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
     </row>
     <row r="50" spans="1:3" x14ac:dyDescent="0.2">
@@ -2504,7 +2504,7 @@
         <v>1</v>
       </c>
       <c r="B50" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
     </row>
     <row r="51" spans="1:3" x14ac:dyDescent="0.2">
@@ -2512,10 +2512,10 @@
         <v>1</v>
       </c>
       <c r="B51" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="C51" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
     </row>
     <row r="52" spans="1:3" x14ac:dyDescent="0.2">
@@ -2523,10 +2523,10 @@
         <v>1</v>
       </c>
       <c r="B52" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="C52" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
     </row>
   </sheetData>

</xml_diff>